<commit_message>
Record live case state: registry, evidence files, and generated reports
Case registry changes from live use (ANV-2026-0004..0011 doc deletions,
ANV-2026-0019 evidence booklet exhibits, _index sequence), refreshed
case_results.xlsx, per-document decision graphs/reports for the
Exhibit P2-P6 evidence set, and regenerated sample-FIR artifacts.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/case_priority_system/case_results.xlsx
+++ b/case_priority_system/case_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,17 +521,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A_K_Kaimal_vs_Sudarsen_Trading_Co_Ltd_And_Anr_on_1_January_1800.PDF</t>
+          <t>03_Exhibit_P2_Bank_Transfers.png</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A.K. Kaimal, Sudarsen Trading Co. Ltd. And Anr.</t>
+          <t>Arjun Nair, Rohan Malhotra</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A.K. Kaimal, a former employee of Chamundy Curing Works, sought to be declared insolvent due to inability to pay two debts. The District Judge dismissed his petition, finding that Kaimal had received a retirement benefit and could not account for its use. The appeal argued that the judge's decision was premature and that the Court should have focused on the insolvency provisions of the Act. The Court allowed the appeal, finding that the judge's dismissal was unjustified and remitted the case for further proceedings.</t>
+          <t>Arjun Nair filed a complaint against Rohan Malhotra for unauthorized bank transfers totaling Rs. 45,00,000 between January and April 2024. The purpose was to deliver vehicles and manage a Whitefield warehouse. The case involves financial disputes related to excise duties and tax assessments.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -540,9 +540,9 @@
 (Neutral, Unbiased Analysis from the Perspective of the Judiciary)
 This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
 ### I. SUBJECT MATTER
-**Parties:** A.K. Kaimal, Sudarsen Trading Co. Ltd. And Anr.
+**Parties:** Arjun Nair, Rohan Malhotra
 **Legal Category:** Excise/Tax
-**Brief Description:** A.K. Kaimal, a former employee of Chamundy Curing Works, sought to be declared insolvent due to inability to pay two debts. The District Judge dismissed his petition, finding that Kaimal had received a retirement benefit and could not account for its use. The appeal argued that the judge's decision was premature and that the Court should have focused on the insolvency provisions of the Act. The Court allowed the appeal, finding that the judge's dismissal was unjustified and remitted the case for further proceedings.
+**Brief Description:** Arjun Nair filed a complaint against Rohan Malhotra for unauthorized bank transfers totaling Rs. 45,00,000 between January and April 2024. The purpose was to deliver vehicles and manage a Whitefield warehouse. The case involves financial disputes related to excise duties and tax assessments.
 **Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = Low
 ### II. CONSTITUTIONAL RIGHTS ENGAGED
 The following constitutional provisions are relevant to this matter:
@@ -599,12 +599,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>case_priority_system/decision_graphs\A_K_Kaimal_vs_Sudarsen_Trading_Co_Ltd_And_Anr_on_1_January_1800_decision_report.md</t>
+          <t>case_priority_system/decision_graphs\03_Exhibit_P2_Bank_Transfers_decision_report.md</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>case_priority_system/decision_graphs\A_K_Kaimal_vs_Sudarsen_Trading_Co_Ltd_And_Anr_on_1_January_1800_decision_report.md</t>
+          <t>case_priority_system/decision_graphs\03_Exhibit_P2_Bank_Transfers_decision_report.md</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -660,17 +660,803 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>case_priority_system\reports\A_K_Kaimal_vs_Sudarsen_Trading_Co_Ltd_And_Anr_on_1_January_1800_report.pdf</t>
+          <t>case_priority_system\reports\03_Exhibit_P2_Bank_Transfers_report.pdf</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>ANV-2026-0010</t>
+          <t>ANV-2026-0019</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>FIR</t>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>04_Exhibit_P3_Disputed_Invoices.png</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kaveri Auto Traders, Prosecution</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Kaveri Auto Traders is accused of fabricating six vehicle invoices. The prosecution disputes their authenticity, citing forensic examination findings. The case involves excise duty and tax disputes.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Kaveri Auto Traders, Prosecution
+**Legal Category:** Excise/Tax
+**Brief Description:** Kaveri Auto Traders is accused of fabricating six vehicle invoices. The prosecution disputes their authenticity, citing forensic examination findings. The case involves excise duty and tax disputes.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = Low
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** Low
+Individuals, small businesses, or parties of comparable standing
+**Constitutional Concern:** Parties are of broadly comparable standing. Article 14 equality concerns are less acute, though the court must still ensure procedural fairness.
+**Recommended Countermeasure:** Standard procedural safeguards apply. The court should proceed with the matter in regular course, without special countermeasures.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Low
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Low Priority**. 
+No urgent constitutional concern is identified. The matter should proceed in regular course. The court remains obligated under Article 14 to ensure that this matter is adjudicated fairly and without inordinate delay, even if it does not warrant special expedition.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
+**RULE 4 — Regulatory/Commercial Matter → Property &amp; Economic Rights:** Articles 14, 19(1)(g), and 300A govern this matter. Priority is based on economic impact and procedural fairness concerns, not life-and-liberty urgency.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Low**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>case_priority_system/decision_graphs\04_Exhibit_P3_Disputed_Invoices_decision_report.md</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>case_priority_system/decision_graphs\04_Exhibit_P3_Disputed_Invoices_decision_report.md</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Excise/Tax</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Non-Violent</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>No Injury</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>[{'article': 'Article 265', 'title': 'Tax Not to be Imposed Save by Authority of Law', 'primary': True, 'why_applies': 'This is a tax case. Article 265 says the government cannot collect any tax unless a law specifically allows it. If the tax was charged without proper legal backing, it must be given back.', 'precedents': []}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other.', 'precedents': []}, {'article': 'Article 19(1)(g)', 'title': 'Right to Practise Any Profession or Carry On Occupation, Trade or Business', 'primary': True, 'why_applies': "This case is about someone's right to run a business, practice a trade, or do a job. Article 19(1)(g) protects that right, but the government can put fair limits on it if the public interest requires it. The court must decide if those limits were reasonable.", 'precedents': []}, {'article': 'Article 300A', 'title': 'Right to Property', 'primary': False, 'why_applies': 'This case involves property or money. Article 300A protects people from losing their property without a lawful reason. The court must check that the proper legal process was followed.', 'precedents': []}, {'article': 'Article 301', 'title': 'Freedom of Trade, Commerce and Intercourse', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': False, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason.", 'precedents': []}]</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}, {'name': 'Doctrine of Reasonable Classification', 'description': 'Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.', 'application': 'Used to test whether differential treatment of litigants or groups is constitutional.'}]</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Category-Specific Analysis — Excise/Tax:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>case_priority_system\reports\04_Exhibit_P3_Disputed_Invoices_report.pdf</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>ANV-2026-0019</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>05_Exhibit_P4_Bank_Statement.png</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HDFC Bank, accused</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>The case involves a transaction summary from a fictional courtroom script, listing financial transactions involving a personal vehicle loan and an online rummy/betting wallet. The accused is accused of misusing funds from these transactions.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** HDFC Bank, accused
+**Legal Category:** General Civil
+**Brief Description:** The case involves a transaction summary from a fictional courtroom script, listing financial transactions involving a personal vehicle loan and an online rummy/betting wallet. The accused is accused of misusing funds from these transactions.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = Low
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[SECONDARY]** Article 39A — Equal Justice and Free Legal Aid**: The State shall secure that the operation of the legal system promotes justice on a basis of equal opportunity, and shall provide free legal aid to ensure that no citizen is denied opportunities to secure justice due to economic or other disability.
+  - Key principles: Free legal aid, Equal opportunity in the legal system, Justice for the economically disadvantaged
+- ****[SECONDARY]** Article 44 — Uniform Civil Code**: The State shall endeavour to secure for the citizens a uniform civil code throughout the territory of India.
+  - Key principles: Uniform civil code for citizens
+- ****[SECONDARY]** Article 51A — Fundamental Duties**: It shall be the duty of every citizen of India to abide by the Constitution and respect its ideals and institutions, to uphold and protect the sovereignty, unity and integrity of India, and to promote harmony and the spirit of common brotherhood.
+  - Key principles: Respect for the Constitution and its institutions, Promotion of harmony and common brotherhood, Protection of public property
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State must ensure that all civil disputes are adjudicated fairly, transparently, and within a reasonable time. Under Article 14, the state guarantees equal access to justice — all litigants are entitled to a fair hearing. The principle of speedy trial (derived from Article 21) requires that even ordinary civil matters be resolved without inordinate delay, though they yield priority to cases involving life and liberty.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** Low
+Individuals, small businesses, or parties of comparable standing
+**Constitutional Concern:** Parties are of broadly comparable standing. Article 14 equality concerns are less acute, though the court must still ensure procedural fairness.
+**Recommended Countermeasure:** Standard procedural safeguards apply. The court should proceed with the matter in regular course, without special countermeasures.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Low
+**Category Rationale:** General civil matters — contracts, consumer disputes, family law, succession — typically engage Article 14's equality guarantee and the right to a fair hearing, but do not involve threats to life, physical safety, or fundamental constitutional rights. They should be processed fairly and without delay, but in regular queue order after more urgent constitutional matters.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Low Priority**. 
+No urgent constitutional concern is identified. The matter should proceed in regular course. The court remains obligated under Article 14 to ensure that this matter is adjudicated fairly and without inordinate delay, even if it does not warrant special expedition.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Low**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>case_priority_system/decision_graphs\05_Exhibit_P4_Bank_Statement_decision_report.md</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>case_priority_system/decision_graphs\05_Exhibit_P4_Bank_Statement_decision_report.md</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>General Civil</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Non-Violent</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>No Injury</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>[{'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other.', 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason.", 'precedents': []}, {'article': 'Article 39A', 'title': 'Equal Justice and Free Legal Aid', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 44', 'title': 'Uniform Civil Code', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 51A', 'title': 'Fundamental Duties', 'primary': False, 'why_applies': '', 'precedents': []}]</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>The State must ensure that all civil disputes are adjudicated fairly, transparently, and within a reasonable time. Under Article 14, the state guarantees equal access to justice — all litigants are entitled to a fair hearing. The principle of speedy trial (derived from Article 21) requires that even ordinary civil matters be resolved without inordinate delay, though they yield priority to cases involving life and liberty.</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}]</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>case_priority_system\reports\05_Exhibit_P4_Bank_Statement_report.pdf</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>ANV-2026-0019</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>06_Exhibit_P5_GST_Certificate.png</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kaveri Auto Traders</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Kaveri Auto Traders is facing a financial dispute related to GST verification. The company's address on invoices does not match the registered GSTIN in departmental records, indicating a potential issue with the authenticity of the GST registration. This case falls under the Excise/Tax category due to the involvement of GST, and it is classified as Financial because it pertains to financial matters.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Kaveri Auto Traders
+**Legal Category:** Excise/Tax
+**Brief Description:** Kaveri Auto Traders is facing a financial dispute related to GST verification. The company's address on invoices does not match the registered GSTIN in departmental records, indicating a potential issue with the authenticity of the GST registration. This case falls under the Excise/Tax category due to the involvement of GST, and it is classified as Financial because it pertains to financial matters.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
+**RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
+**RULE 4 — Regulatory/Commercial Matter → Property &amp; Economic Rights:** Articles 14, 19(1)(g), and 300A govern this matter. Priority is based on economic impact and procedural fairness concerns, not life-and-liberty urgency.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Medium**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>case_priority_system/decision_graphs\06_Exhibit_P5_GST_Certificate_decision_report.md</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>case_priority_system/decision_graphs\06_Exhibit_P5_GST_Certificate_decision_report.md</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Excise/Tax</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Non-Violent</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>No Injury</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>[{'article': 'Article 265', 'title': 'Tax Not to be Imposed Save by Authority of Law', 'primary': True, 'why_applies': 'This is a tax case. Article 265 says the government cannot collect any tax unless a law specifically allows it. If the tax was charged without proper legal backing, it must be given back.', 'precedents': []}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other. One side is much more powerful than the other — a government body, a large company, or someone with political influence. Article 14 requires the court to make sure the weaker party is not overpowered.', 'precedents': []}, {'article': 'Article 19(1)(g)', 'title': 'Right to Practise Any Profession or Carry On Occupation, Trade or Business', 'primary': True, 'why_applies': "This case is about someone's right to run a business, practice a trade, or do a job. Article 19(1)(g) protects that right, but the government can put fair limits on it if the public interest requires it. The court must decide if those limits were reasonable.", 'precedents': []}, {'article': 'Article 300A', 'title': 'Right to Property', 'primary': False, 'why_applies': 'This case involves property or money. Article 300A protects people from losing their property without a lawful reason. The court must check that the proper legal process was followed.', 'precedents': []}, {'article': 'Article 301', 'title': 'Freedom of Trade, Commerce and Intercourse', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': False, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason.", 'precedents': []}]</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}, {'name': 'Doctrine of Reasonable Classification', 'description': 'Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.', 'application': 'Used to test whether differential treatment of litigants or groups is constitutional.'}]</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
+**Category-Specific Analysis — Excise/Tax:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>case_priority_system\reports\06_Exhibit_P5_GST_Certificate_report.pdf</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>ANV-2026-0019</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>07_Exhibit_P6_Forensic_Report.png</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kaveri Auto Traders</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Kaveri Auto Traders is accused of fabricating six invoices attributed to them. The case involves financial disputes related to excise duties and GST, as the invoices were retrospectively dated and used in a courtroom script to support the fabricated claim.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Kaveri Auto Traders
+**Legal Category:** Excise/Tax
+**Brief Description:** Kaveri Auto Traders is accused of fabricating six invoices attributed to them. The case involves financial disputes related to excise duties and GST, as the invoices were retrospectively dated and used in a courtroom script to support the fabricated claim.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = Low
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** Low
+Individuals, small businesses, or parties of comparable standing
+**Constitutional Concern:** Parties are of broadly comparable standing. Article 14 equality concerns are less acute, though the court must still ensure procedural fairness.
+**Recommended Countermeasure:** Standard procedural safeguards apply. The court should proceed with the matter in regular course, without special countermeasures.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Low
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Low Priority**. 
+No urgent constitutional concern is identified. The matter should proceed in regular course. The court remains obligated under Article 14 to ensure that this matter is adjudicated fairly and without inordinate delay, even if it does not warrant special expedition.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
+**RULE 4 — Regulatory/Commercial Matter → Property &amp; Economic Rights:** Articles 14, 19(1)(g), and 300A govern this matter. Priority is based on economic impact and procedural fairness concerns, not life-and-liberty urgency.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Low**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>case_priority_system/decision_graphs\07_Exhibit_P6_Forensic_Report_decision_report.md</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>case_priority_system/decision_graphs\07_Exhibit_P6_Forensic_Report_decision_report.md</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Excise/Tax</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Non-Violent</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>No Injury</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>[{'article': 'Article 265', 'title': 'Tax Not to be Imposed Save by Authority of Law', 'primary': True, 'why_applies': 'This is a tax case. Article 265 says the government cannot collect any tax unless a law specifically allows it. If the tax was charged without proper legal backing, it must be given back.', 'precedents': []}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other.', 'precedents': []}, {'article': 'Article 19(1)(g)', 'title': 'Right to Practise Any Profession or Carry On Occupation, Trade or Business', 'primary': True, 'why_applies': "This case is about someone's right to run a business, practice a trade, or do a job. Article 19(1)(g) protects that right, but the government can put fair limits on it if the public interest requires it. The court must decide if those limits were reasonable.", 'precedents': []}, {'article': 'Article 300A', 'title': 'Right to Property', 'primary': False, 'why_applies': 'This case involves property or money. Article 300A protects people from losing their property without a lawful reason. The court must check that the proper legal process was followed.', 'precedents': []}, {'article': 'Article 301', 'title': 'Freedom of Trade, Commerce and Intercourse', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': False, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason.", 'precedents': []}]</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}, {'name': 'Doctrine of Reasonable Classification', 'description': 'Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.', 'application': 'Used to test whether differential treatment of litigants or groups is constitutional.'}]</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Category-Specific Analysis — Excise/Tax:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>case_priority_system\reports\07_Exhibit_P6_Forensic_Report_report.pdf</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>ANV-2026-0019</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>09_Evidence_Booklet.pdf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>STATE (ON COMPLAINT OF ARJUN NAIR), ROHAN MALHOTRA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>STATE, on the complaint of ARJUN NAIR, seeks to hold ROHAN MALHOTRA liable for breach of a partnership agreement. The dispute centers around disputed invoices and bank transfer receipts. The case raises questions under Article 21 (right to life and personal liberty) and Article 14 (equality before law). The relief sought is for the enforcement of the partnership agreement and payment of dues.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** STATE (ON COMPLAINT OF ARJUN NAIR), ROHAN MALHOTRA
+**Legal Category:** Constitutional/Writ
+**Brief Description:** STATE, on the complaint of ARJUN NAIR, seeks to hold ROHAN MALHOTRA liable for breach of a partnership agreement. The dispute centers around disputed invoices and bank transfer receipts. The case raises questions under Article 21 (right to life and personal liberty) and Article 14 (equality before law). The relief sought is for the enforcement of the partnership agreement and payment of dues.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 32 — Remedies for Enforcement of Fundamental Rights**: The right to move the Supreme Court for the enforcement of fundamental rights is guaranteed.
+  - Key principles: Right to constitutional remedies, Writ jurisdiction of Supreme Court, Enforcement of fundamental rights
+- ****[PRIMARY]** Article 226 — Power of High Courts to Issue Certain Writs**: Every High Court shall have power to issue directions, orders, or writs for enforcement of fundamental rights and for any other purpose.
+  - Key principles: Writ jurisdiction of High Courts, Judicial review of state action, Enforcement of legal rights
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[SECONDARY]** Article 227 — Power of Superintendence of High Courts**: Every High Court shall have superintendence over all courts and tribunals within its jurisdiction, and may call for returns, make rules, and settle forms to secure the proper administration of justice.
+  - Key principles: Superintendence over subordinate courts and tribunals, Administration of justice
+- ****[SECONDARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
+  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
+- ****[SECONDARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
+  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
+- ****[SECONDARY]** Article 51A — Fundamental Duties**: It shall be the duty of every citizen of India to abide by the Constitution and respect its ideals and institutions, to uphold and protect the sovereignty, unity and integrity of India, and to promote harmony and the spirit of common brotherhood.
+  - Key principles: Respect for the Constitution and its institutions, Promotion of harmony and common brotherhood, Protection of public property
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State, through the judiciary, is the ultimate guardian of fundamental rights. Under Articles 32 and 226, the High Courts and Supreme Court have a constitutional duty to protect citizens against arbitrary state action, violations of fundamental rights, and jurisdictional errors by subordinate tribunals. These cases often involve the very legitimacy of state action and require careful, principled consideration.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Basic Structure**: The Parliament cannot amend the Constitution to destroy its basic features such as supremacy of the Constitution, rule of law, and judicial review.
+  - Application to this case: Applicable to cases involving constitutional amendments or executive actions affecting foundational principles.
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Colourable Legislation**: If the legislature lacks the competence to enact a law directly, it cannot do indirectly what it cannot do directly — such camouflage is struck down.
+  - Application to this case: Applicable where a statute purports to do one thing but in substance does another outside legislative competence.
+- **Doctrine of Harmonious Construction**: Where two constitutional provisions conflict, they should be interpreted so that both are given effect rather than one nullifying the other.
+  - Application to this case: Used when Articles or statutory provisions appear to overlap or clash.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Constitutional writ matters directly engage fundamental rights and the rule of law. Cases involving imminent threats to life or liberty (habeas corpus) warrant the highest priority. Cases challenging administrative or quasi-judicial orders should receive priority proportionate to the gravity of the rights violation alleged and the urgency of the relief sought.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
+**RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
+**RULE 4 — Constitutional/Writ Matter → Article 32/226 Jurisdiction:** The court's constitutional writ jurisdiction is engaged. Priority depends on the nature of the right sought to be enforced.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Medium**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>case_priority_system/decision_graphs\09_Evidence_Booklet_decision_report.md</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>case_priority_system/decision_graphs\09_Evidence_Booklet_decision_report.md</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Constitutional/Writ</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Non-Violent</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>No Injury</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>[{'article': 'Article 32', 'title': 'Remedies for Enforcement of Fundamental Rights', 'primary': True, 'why_applies': 'This case has been filed directly in the Supreme Court. Article 32 gives every citizen the right to go to the Supreme Court if their basic rights are being taken away. It is the tool that makes sure all the other rights actually work.', 'precedents': []}, {'article': 'Article 226', 'title': 'Power of High Courts to Issue Certain Writs', 'primary': True, 'why_applies': 'This case has been filed in a High Court. Article 226 gives High Courts the power to order the government to follow the law. If a government body does something illegal, this article lets citizens ask the court to step in and fix it.', 'precedents': []}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other. One side is much more powerful than the other — a government body, a large company, or someone with political influence. Article 14 requires the court to make sure the weaker party is not overpowered.', 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason.", 'precedents': []}, {'article': 'Article 227', 'title': 'Power of Superintendence of High Courts', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 22', 'title': 'Protection Against Arrest and Detention', 'primary': False, 'why_applies': 'Someone has been arrested. Article 22 says they must be told why, allowed to talk to a lawyer, and not kept in jail forever without a proper hearing. It protects people from being locked up without reason.', 'precedents': []}, {'article': 'Article 20', 'title': 'Protection in Respect of Conviction for Offences', 'primary': False, 'why_applies': 'This is a criminal case. Article 20 protects the accused person from being treated unfairly. It says: you cannot be punished for something that was not a crime when you did it, you cannot be tried twice for the same offence, and you cannot be forced to confess.', 'precedents': []}, {'article': 'Article 51A', 'title': 'Fundamental Duties', 'primary': False, 'why_applies': '', 'precedents': []}]</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>The State, through the judiciary, is the ultimate guardian of fundamental rights. Under Articles 32 and 226, the High Courts and Supreme Court have a constitutional duty to protect citizens against arbitrary state action, violations of fundamental rights, and jurisdictional errors by subordinate tribunals. These cases often involve the very legitimacy of state action and require careful, principled consideration.</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>[{'name': 'Doctrine of Basic Structure', 'description': 'The Parliament cannot amend the Constitution to destroy its basic features such as supremacy of the Constitution, rule of law, and judicial review.', 'application': 'Applicable to cases involving constitutional amendments or executive actions affecting foundational principles.'}, {'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}, {'name': 'Doctrine of Colourable Legislation', 'description': 'If the legislature lacks the competence to enact a law directly, it cannot do indirectly what it cannot do directly — such camouflage is struck down.', 'application': 'Applicable where a statute purports to do one thing but in substance does another outside legislative competence.'}, {'name': 'Doctrine of Harmonious Construction', 'description': 'Where two constitutional provisions conflict, they should be interpreted so that both are given effect rather than one nullifying the other.', 'application': 'Used when Articles or statutory provisions appear to overlap or clash.'}]</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
+**Category-Specific Analysis — Constitutional/Writ:** Writ matters directly engage the court's constitutional jurisdiction under Articles 32 and 226. The priority should reflect the nature of the right sought to be enforced — habeas corpus (life/liberty) cases require the highest priority.</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>case_priority_system\reports\09_Evidence_Booklet_report.pdf</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>ANV-2026-0019</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Other</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(case-registry): add ANV-2026-0025 missing child case registry dossier and documents
</commit_message>
<xml_diff>
--- a/case_priority_system/case_results.xlsx
+++ b/case_priority_system/case_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="153">
   <si>
     <t>Case_File</t>
   </si>
@@ -97,6 +97,30 @@
     <t>[WHOLE CASE] Evidence Booklet — State vs Kaveri Auto Traders</t>
   </si>
   <si>
+    <t>Evidence_01_Incident_Report_and_Timeline.pdf</t>
+  </si>
+  <si>
+    <t>Evidence_02_CCTV_Review_Log.pdf</t>
+  </si>
+  <si>
+    <t>Evidence_03_Shop_Audio_Transcript_SIMULATED.pdf</t>
+  </si>
+  <si>
+    <t>Evidence_04_Witness_Statements_SIMULATED.pdf</t>
+  </si>
+  <si>
+    <t>Evidence_05_Traffic_Camera_Note.pdf</t>
+  </si>
+  <si>
+    <t>Evidence_06_Interview_Records_SIMULATED.pdf</t>
+  </si>
+  <si>
+    <t>Evidence_08_Evidence_Register_and_Corroboration.pdf</t>
+  </si>
+  <si>
+    <t>[WHOLE CASE] Missing case</t>
+  </si>
+  <si>
     <t>Arjun Nair, Rohan Malhotra</t>
   </si>
   <si>
@@ -115,6 +139,30 @@
     <t>Arjun Nair, Rohan Malhotra, Kaveri Auto Traders, Prosecution, HDFC Bank, accused, STATE (ON COMPLAINT OF ARJUN NAIR)</t>
   </si>
   <si>
+    <t>Meera Rao, Nisha Rao</t>
+  </si>
+  <si>
+    <t>Meera, Unknown Person in a Yellow Shirt</t>
+  </si>
+  <si>
+    <t>Unknown parties involved in a fictional scenario</t>
+  </si>
+  <si>
+    <t>Child, Adult, Shop Employee, Security Guard, Balloon Vendor</t>
+  </si>
+  <si>
+    <t>Meera, Suspect</t>
+  </si>
+  <si>
+    <t>Nisha Rao, Meera, Arun</t>
+  </si>
+  <si>
+    <t>Party A, Party B</t>
+  </si>
+  <si>
+    <t>Meera Rao, Nisha Rao, Meera, Unknown Person in a Yellow Shirt, Unknown parties involved in a fictional scenario, Child, Adult, Shop Employee, Security Guard, Balloon Vendor, Suspect, Arun, Party A, Party B</t>
+  </si>
+  <si>
     <t>Arjun Nair filed a complaint against Rohan Malhotra for unauthorized bank transfers totaling Rs. 45,00,000 between January and April 2024. The purpose was to deliver vehicles and manage a Whitefield warehouse. The case involves financial disputes related to excise duties and tax assessments.</t>
   </si>
   <si>
@@ -134,6 +182,30 @@
   </si>
   <si>
     <t>This case file brings together 6 documents (6 × Other) and is assessed as a single matter of Excise/Tax with no injury indicated. The evidence on record consists of “03_Exhibit_P2_Bank_Transfers.png” (Other; Excise/Tax; assessed Low priority); “04_Exhibit_P3_Disputed_Invoices.png” (Other; Excise/Tax; assessed Low priority); “05_Exhibit_P4_Bank_Statement.png” (Other; General Civil; assessed Low priority); “06_Exhibit_P5_GST_Certificate.png” (Other; Excise/Tax; assessed Medium priority); “07_Exhibit_P6_Forensic_Report.png” (Other; Excise/Tax; assessed Low priority); “09_Evidence_Booklet.pdf” (Other; Constitutional/Writ; assessed Medium priority). Cross-comparison finds 4 corroborating links between the documents (shared dates, places or parties), which strengthens the consistency of the record. For example, “03_Exhibit_P2_Bank_Transfers.png” and “09_Evidence_Booklet.pdf” share parties. “05_Exhibit_P4_Bank_Statement.png” currently stands alone — no other document shares a date, place or party with it, so further supporting evidence would strengthen the case.</t>
+  </si>
+  <si>
+    <t>Meera Rao, a 9-year-old child, was reported missing from Lakeview Community Park on September 28, 2026. Her mother, Nisha Rao, reported her last seen near the play area at 18:18. The police were notified at 18:24 and a fictional FIR was recorded. The case involves a child in danger, engaging Article 21 of the Indian Constitution, which protects life and personal liberty.</t>
+  </si>
+  <si>
+    <t>Meera, a vulnerable elderly woman, was allegedly assaulted by an unknown person in a yellow shirt. The dispute centers around the assault and the unknown assailant's identity. This case engages Article 21 (right to life and personal liberty) and Article 14 (equality before law). The case falls under the Criminal/Violent category as it involves a serious injury and the need to establish the identity of the assailant, which is crucial for justice and protection.</t>
+  </si>
+  <si>
+    <t>In a fictional scenario, no parties are identified. The dispute involves a fictional conversation recorded in a shop, with no real harm or legal issues. The case seeks clarification on the rights of parties in a fictional scenario and does not involve any real legal disputes. The case falls under General Civil as it deals with a non-violent, non-injury scenario without any real parties or legal issues.</t>
+  </si>
+  <si>
+    <t>In a fictional scenario, a child was allegedly abducted near a park. The shop employee heard raised voices outside the shop, but could not identify the speakers. The security guard noticed an adult in a yellow shirt near the service road. The balloon vendor saw a child near the park path. The case involves a child's safety and the alleged abduction, engaging Article 21 of the Indian Constitution, which protects life and personal liberty.</t>
+  </si>
+  <si>
+    <t>Meera, a minor, is alleged to have been kidnapped and assaulted by a suspect. The dispute centers around the authenticity of a fictional traffic-camera footage that may have provided clues to the suspect's movements. The case raises questions under Article 21 (right to life and personal liberty) and Article 14 (equality before law). The case falls under the Criminal/Violent category due to the serious injury and vulnerability of the minor Meera.</t>
+  </si>
+  <si>
+    <t>Nisha Rao, the mother, reported that her daughter Meera was last seen near the play area at 6:18 PM. Meera was not found and Nisha called for help. Arun, a person of interest, claims he did not take the child. The case involves a missing child, potential criminal activity, and the right to life and personal liberty under Article 21 of the Indian Constitution.</t>
+  </si>
+  <si>
+    <t>In this fictional scenario, Party A and Party B are involved in a violent dispute over property rights. The dispute escalated to physical harm, with Party B allegedly assaulting Party A. The case raises questions under Article 21 (right to life and personal liberty) and Article 14 (equality before law). The case falls under the Criminal/Violent category as it involves a major injury and a power imbalance.</t>
+  </si>
+  <si>
+    <t>This case file brings together 7 documents (FIR, 6 × Other) and is assessed as a single matter of Constitutional/Writ with no injury indicated, involving vulnerable parties. The evidence on record consists of “Evidence_01_Incident_Report_and_Timeline.pdf” (FIR; Constitutional/Writ; assessed Medium priority); “Evidence_02_CCTV_Review_Log.pdf” (Other; Constitutional/Writ; assessed Medium priority); “Evidence_03_Shop_Audio_Transcript_SIMULATED.pdf” (Other; General Civil; assessed Medium priority); “Evidence_04_Witness_Statements_SIMULATED.pdf” (Other; Constitutional/Writ; assessed Medium priority); “Evidence_05_Traffic_Camera_Note.pdf” (Other; Constitutional/Writ; assessed Medium priority); “Evidence_06_Interview_Records_SIMULATED.pdf” (Other; Excise/Tax; assessed Medium priority); “Evidence_08_Evidence_Register_and_Corroboration.pdf” (Other; Constitutional/Writ; assessed Medium priority). Cross-comparison finds 4 corroborating links between the documents (shared dates, places or parties), which strengthens the consistency of the record. For example, “Evidence_01_Incident_Report_and_Timeline.pdf” and “Evidence_06_Interview_Records_SIMULATED.pdf” share parties. “Evidence_03_Shop_Audio_Transcript_SIMULATED.pdf”, “Evidence_04_Witness_Statements_SIMULATED.pdf”, “Evidence_08_Evidence_Register_and_Corroboration.pdf” currently stand alone — no other document shares a date, place or party with them, so further supporting evidence would strengthen the case.</t>
   </si>
   <si>
     <t>## STATE'S CONSTITUTIONAL ASSESSMENT
@@ -518,6 +590,472 @@
 The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
   </si>
   <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Meera Rao, Nisha Rao
+**Legal Category:** Constitutional/Writ
+**Brief Description:** Meera Rao, a 9-year-old child, was reported missing from Lakeview Community Park on September 28, 2026. Her mother, Nisha Rao, reported her last seen near the play area at 18:18. The police were notified at 18:24 and a fictional FIR was recorded. The case involves a child in danger, engaging Article 21 of the Indian Constitution, which protects life and personal liberty.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = High, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 32 — Remedies for Enforcement of Fundamental Rights**: The right to move the Supreme Court for the enforcement of fundamental rights is guaranteed.
+  - Key principles: Right to constitutional remedies, Writ jurisdiction of Supreme Court, Enforcement of fundamental rights
+- ****[PRIMARY]** Article 226 — Power of High Courts to Issue Certain Writs**: Every High Court shall have power to issue directions, orders, or writs for enforcement of fundamental rights and for any other purpose.
+  - Key principles: Writ jurisdiction of High Courts, Judicial review of state action, Enforcement of legal rights
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[SECONDARY]** Article 227 — Power of Superintendence of High Courts**: Every High Court shall have superintendence over all courts and tribunals within its jurisdiction, and may call for returns, make rules, and settle forms to secure the proper administration of justice.
+  - Key principles: Superintendence over subordinate courts and tribunals, Administration of justice
+- ****[SECONDARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
+  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
+- ****[SECONDARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
+  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
+- ****[SECONDARY]** Article 51A — Fundamental Duties**: It shall be the duty of every citizen of India to abide by the Constitution and respect its ideals and institutions, to uphold and protect the sovereignty, unity and integrity of India, and to promote harmony and the spirit of common brotherhood.
+  - Key principles: Respect for the Constitution and its institutions, Promotion of harmony and common brotherhood, Protection of public property
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State, through the judiciary, is the ultimate guardian of fundamental rights. Under Articles 32 and 226, the High Courts and Supreme Court have a constitutional duty to protect citizens against arbitrary state action, violations of fundamental rights, and jurisdictional errors by subordinate tribunals. These cases often involve the very legitimacy of state action and require careful, principled consideration.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** High
+This indicates: ['Minors / Children', 'Pregnant Women', 'Elderly / Senior Citizens', 'Disabled Persons', 'Scheduled Castes (SC)', 'Scheduled Tribes (ST)', 'Other Backward Classes (OBC)', 'Adivasis / Tribals', 'Dalits', 'Economically Weaker Sections (EWS)', 'Below Poverty Line (BPL)', 'Daily Wage Workers', 'Agricultural Labourers', 'Domestic Workers', 'Migrant Workers', 'Unorganised Sector Workers', 'Bonded Labourers', 'Sex Workers', 'Human Trafficking Survivors', 'Refugees / Asylum Seekers', 'Homeless Persons', 'Orphans', 'Single Mothers / Widows', 'Persons in Custody', 'Victims of Domestic Violence', 'Victims of Sexual Assault', 'Victims of Torture']
+**Constitutional Protection:** Articles 14, 15, 15(3), 15(4), 15(5), 16(4), 17, 23, 24, 39, 39A, 41, 46, and the Directive Principles under Part IV mandate special protection for vulnerable groups. The Doctrine of Parens Patriae obligates the state to act as guardian for those who cannot protect themselves.
+**Judicial Duty:** The court must adopt a protective, sensitised approach. Vulnerable litigants are entitled to: (a) in-camera proceedings where appropriate, (b) assistance of counsel if unrepresented, (c) protection from intimidation, (d) expedited hearings to prevent secondary trauma, and (e) rehabilitation and compensation directions where applicable.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Basic Structure**: The Parliament cannot amend the Constitution to destroy its basic features such as supremacy of the Constitution, rule of law, and judicial review.
+  - Application to this case: Applicable to cases involving constitutional amendments or executive actions affecting foundational principles.
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Colourable Legislation**: If the legislature lacks the competence to enact a law directly, it cannot do indirectly what it cannot do directly — such camouflage is struck down.
+  - Application to this case: Applicable where a statute purports to do one thing but in substance does another outside legislative competence.
+- **Doctrine of Harmonious Construction**: Where two constitutional provisions conflict, they should be interpreted so that both are given effect rather than one nullifying the other.
+  - Application to this case: Used when Articles or statutory provisions appear to overlap or clash.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Constitutional writ matters directly engage fundamental rights and the rule of law. Cases involving imminent threats to life or liberty (habeas corpus) warrant the highest priority. Cases challenging administrative or quasi-judicial orders should receive priority proportionate to the gravity of the rights violation alleged and the urgency of the relief sought.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Meera, Unknown Person in a Yellow Shirt
+**Legal Category:** Constitutional/Writ
+**Brief Description:** Meera, a vulnerable elderly woman, was allegedly assaulted by an unknown person in a yellow shirt. The dispute centers around the assault and the unknown assailant's identity. This case engages Article 21 (right to life and personal liberty) and Article 14 (equality before law). The case falls under the Criminal/Violent category as it involves a serious injury and the need to establish the identity of the assailant, which is crucial for justice and protection.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 32 — Remedies for Enforcement of Fundamental Rights**: The right to move the Supreme Court for the enforcement of fundamental rights is guaranteed.
+  - Key principles: Right to constitutional remedies, Writ jurisdiction of Supreme Court, Enforcement of fundamental rights
+- ****[PRIMARY]** Article 226 — Power of High Courts to Issue Certain Writs**: Every High Court shall have power to issue directions, orders, or writs for enforcement of fundamental rights and for any other purpose.
+  - Key principles: Writ jurisdiction of High Courts, Judicial review of state action, Enforcement of legal rights
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[SECONDARY]** Article 227 — Power of Superintendence of High Courts**: Every High Court shall have superintendence over all courts and tribunals within its jurisdiction, and may call for returns, make rules, and settle forms to secure the proper administration of justice.
+  - Key principles: Superintendence over subordinate courts and tribunals, Administration of justice
+- ****[SECONDARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
+  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
+- ****[SECONDARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
+  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
+- ****[SECONDARY]** Article 51A — Fundamental Duties**: It shall be the duty of every citizen of India to abide by the Constitution and respect its ideals and institutions, to uphold and protect the sovereignty, unity and integrity of India, and to promote harmony and the spirit of common brotherhood.
+  - Key principles: Respect for the Constitution and its institutions, Promotion of harmony and common brotherhood, Protection of public property
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State, through the judiciary, is the ultimate guardian of fundamental rights. Under Articles 32 and 226, the High Courts and Supreme Court have a constitutional duty to protect citizens against arbitrary state action, violations of fundamental rights, and jurisdictional errors by subordinate tribunals. These cases often involve the very legitimacy of state action and require careful, principled consideration.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Basic Structure**: The Parliament cannot amend the Constitution to destroy its basic features such as supremacy of the Constitution, rule of law, and judicial review.
+  - Application to this case: Applicable to cases involving constitutional amendments or executive actions affecting foundational principles.
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Colourable Legislation**: If the legislature lacks the competence to enact a law directly, it cannot do indirectly what it cannot do directly — such camouflage is struck down.
+  - Application to this case: Applicable where a statute purports to do one thing but in substance does another outside legislative competence.
+- **Doctrine of Harmonious Construction**: Where two constitutional provisions conflict, they should be interpreted so that both are given effect rather than one nullifying the other.
+  - Application to this case: Used when Articles or statutory provisions appear to overlap or clash.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Constitutional writ matters directly engage fundamental rights and the rule of law. Cases involving imminent threats to life or liberty (habeas corpus) warrant the highest priority. Cases challenging administrative or quasi-judicial orders should receive priority proportionate to the gravity of the rights violation alleged and the urgency of the relief sought.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Unknown parties involved in a fictional scenario
+**Legal Category:** General Civil
+**Brief Description:** In a fictional scenario, no parties are identified. The dispute involves a fictional conversation recorded in a shop, with no real harm or legal issues. The case seeks clarification on the rights of parties in a fictional scenario and does not involve any real legal disputes. The case falls under General Civil as it deals with a non-violent, non-injury scenario without any real parties or legal issues.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[SECONDARY]** Article 39A — Equal Justice and Free Legal Aid**: The State shall secure that the operation of the legal system promotes justice on a basis of equal opportunity, and shall provide free legal aid to ensure that no citizen is denied opportunities to secure justice due to economic or other disability.
+  - Key principles: Free legal aid, Equal opportunity in the legal system, Justice for the economically disadvantaged
+- ****[SECONDARY]** Article 44 — Uniform Civil Code**: The State shall endeavour to secure for the citizens a uniform civil code throughout the territory of India.
+  - Key principles: Uniform civil code for citizens
+- ****[SECONDARY]** Article 51A — Fundamental Duties**: It shall be the duty of every citizen of India to abide by the Constitution and respect its ideals and institutions, to uphold and protect the sovereignty, unity and integrity of India, and to promote harmony and the spirit of common brotherhood.
+  - Key principles: Respect for the Constitution and its institutions, Promotion of harmony and common brotherhood, Protection of public property
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State must ensure that all civil disputes are adjudicated fairly, transparently, and within a reasonable time. Under Article 14, the state guarantees equal access to justice — all litigants are entitled to a fair hearing. The principle of speedy trial (derived from Article 21) requires that even ordinary civil matters be resolved without inordinate delay, though they yield priority to cases involving life and liberty.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** General civil matters — contracts, consumer disputes, family law, succession — typically engage Article 14's equality guarantee and the right to a fair hearing, but do not involve threats to life, physical safety, or fundamental constitutional rights. They should be processed fairly and without delay, but in regular queue order after more urgent constitutional matters.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Child, Adult, Shop Employee, Security Guard, Balloon Vendor
+**Legal Category:** Constitutional/Writ
+**Brief Description:** In a fictional scenario, a child was allegedly abducted near a park. The shop employee heard raised voices outside the shop, but could not identify the speakers. The security guard noticed an adult in a yellow shirt near the service road. The balloon vendor saw a child near the park path. The case involves a child's safety and the alleged abduction, engaging Article 21 of the Indian Constitution, which protects life and personal liberty.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = High, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 32 — Remedies for Enforcement of Fundamental Rights**: The right to move the Supreme Court for the enforcement of fundamental rights is guaranteed.
+  - Key principles: Right to constitutional remedies, Writ jurisdiction of Supreme Court, Enforcement of fundamental rights
+- ****[PRIMARY]** Article 226 — Power of High Courts to Issue Certain Writs**: Every High Court shall have power to issue directions, orders, or writs for enforcement of fundamental rights and for any other purpose.
+  - Key principles: Writ jurisdiction of High Courts, Judicial review of state action, Enforcement of legal rights
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[SECONDARY]** Article 227 — Power of Superintendence of High Courts**: Every High Court shall have superintendence over all courts and tribunals within its jurisdiction, and may call for returns, make rules, and settle forms to secure the proper administration of justice.
+  - Key principles: Superintendence over subordinate courts and tribunals, Administration of justice
+- ****[SECONDARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
+  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
+- ****[SECONDARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
+  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
+- ****[SECONDARY]** Article 51A — Fundamental Duties**: It shall be the duty of every citizen of India to abide by the Constitution and respect its ideals and institutions, to uphold and protect the sovereignty, unity and integrity of India, and to promote harmony and the spirit of common brotherhood.
+  - Key principles: Respect for the Constitution and its institutions, Promotion of harmony and common brotherhood, Protection of public property
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State, through the judiciary, is the ultimate guardian of fundamental rights. Under Articles 32 and 226, the High Courts and Supreme Court have a constitutional duty to protect citizens against arbitrary state action, violations of fundamental rights, and jurisdictional errors by subordinate tribunals. These cases often involve the very legitimacy of state action and require careful, principled consideration.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** High
+This indicates: ['Minors / Children', 'Pregnant Women', 'Elderly / Senior Citizens', 'Disabled Persons', 'Scheduled Castes (SC)', 'Scheduled Tribes (ST)', 'Other Backward Classes (OBC)', 'Adivasis / Tribals', 'Dalits', 'Economically Weaker Sections (EWS)', 'Below Poverty Line (BPL)', 'Daily Wage Workers', 'Agricultural Labourers', 'Domestic Workers', 'Migrant Workers', 'Unorganised Sector Workers', 'Bonded Labourers', 'Sex Workers', 'Human Trafficking Survivors', 'Refugees / Asylum Seekers', 'Homeless Persons', 'Orphans', 'Single Mothers / Widows', 'Persons in Custody', 'Victims of Domestic Violence', 'Victims of Sexual Assault', 'Victims of Torture']
+**Constitutional Protection:** Articles 14, 15, 15(3), 15(4), 15(5), 16(4), 17, 23, 24, 39, 39A, 41, 46, and the Directive Principles under Part IV mandate special protection for vulnerable groups. The Doctrine of Parens Patriae obligates the state to act as guardian for those who cannot protect themselves.
+**Judicial Duty:** The court must adopt a protective, sensitised approach. Vulnerable litigants are entitled to: (a) in-camera proceedings where appropriate, (b) assistance of counsel if unrepresented, (c) protection from intimidation, (d) expedited hearings to prevent secondary trauma, and (e) rehabilitation and compensation directions where applicable.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Basic Structure**: The Parliament cannot amend the Constitution to destroy its basic features such as supremacy of the Constitution, rule of law, and judicial review.
+  - Application to this case: Applicable to cases involving constitutional amendments or executive actions affecting foundational principles.
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Colourable Legislation**: If the legislature lacks the competence to enact a law directly, it cannot do indirectly what it cannot do directly — such camouflage is struck down.
+  - Application to this case: Applicable where a statute purports to do one thing but in substance does another outside legislative competence.
+- **Doctrine of Harmonious Construction**: Where two constitutional provisions conflict, they should be interpreted so that both are given effect rather than one nullifying the other.
+  - Application to this case: Used when Articles or statutory provisions appear to overlap or clash.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Constitutional writ matters directly engage fundamental rights and the rule of law. Cases involving imminent threats to life or liberty (habeas corpus) warrant the highest priority. Cases challenging administrative or quasi-judicial orders should receive priority proportionate to the gravity of the rights violation alleged and the urgency of the relief sought.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Meera, Suspect
+**Legal Category:** Constitutional/Writ
+**Brief Description:** Meera, a minor, is alleged to have been kidnapped and assaulted by a suspect. The dispute centers around the authenticity of a fictional traffic-camera footage that may have provided clues to the suspect's movements. The case raises questions under Article 21 (right to life and personal liberty) and Article 14 (equality before law). The case falls under the Criminal/Violent category due to the serious injury and vulnerability of the minor Meera.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 32 — Remedies for Enforcement of Fundamental Rights**: The right to move the Supreme Court for the enforcement of fundamental rights is guaranteed.
+  - Key principles: Right to constitutional remedies, Writ jurisdiction of Supreme Court, Enforcement of fundamental rights
+- ****[PRIMARY]** Article 226 — Power of High Courts to Issue Certain Writs**: Every High Court shall have power to issue directions, orders, or writs for enforcement of fundamental rights and for any other purpose.
+  - Key principles: Writ jurisdiction of High Courts, Judicial review of state action, Enforcement of legal rights
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[SECONDARY]** Article 227 — Power of Superintendence of High Courts**: Every High Court shall have superintendence over all courts and tribunals within its jurisdiction, and may call for returns, make rules, and settle forms to secure the proper administration of justice.
+  - Key principles: Superintendence over subordinate courts and tribunals, Administration of justice
+- ****[SECONDARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
+  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
+- ****[SECONDARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
+  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
+- ****[SECONDARY]** Article 51A — Fundamental Duties**: It shall be the duty of every citizen of India to abide by the Constitution and respect its ideals and institutions, to uphold and protect the sovereignty, unity and integrity of India, and to promote harmony and the spirit of common brotherhood.
+  - Key principles: Respect for the Constitution and its institutions, Promotion of harmony and common brotherhood, Protection of public property
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State, through the judiciary, is the ultimate guardian of fundamental rights. Under Articles 32 and 226, the High Courts and Supreme Court have a constitutional duty to protect citizens against arbitrary state action, violations of fundamental rights, and jurisdictional errors by subordinate tribunals. These cases often involve the very legitimacy of state action and require careful, principled consideration.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Basic Structure**: The Parliament cannot amend the Constitution to destroy its basic features such as supremacy of the Constitution, rule of law, and judicial review.
+  - Application to this case: Applicable to cases involving constitutional amendments or executive actions affecting foundational principles.
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Colourable Legislation**: If the legislature lacks the competence to enact a law directly, it cannot do indirectly what it cannot do directly — such camouflage is struck down.
+  - Application to this case: Applicable where a statute purports to do one thing but in substance does another outside legislative competence.
+- **Doctrine of Harmonious Construction**: Where two constitutional provisions conflict, they should be interpreted so that both are given effect rather than one nullifying the other.
+  - Application to this case: Used when Articles or statutory provisions appear to overlap or clash.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Constitutional writ matters directly engage fundamental rights and the rule of law. Cases involving imminent threats to life or liberty (habeas corpus) warrant the highest priority. Cases challenging administrative or quasi-judicial orders should receive priority proportionate to the gravity of the rights violation alleged and the urgency of the relief sought.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Nisha Rao, Meera, Arun
+**Legal Category:** Excise/Tax
+**Brief Description:** Nisha Rao, the mother, reported that her daughter Meera was last seen near the play area at 6:18 PM. Meera was not found and Nisha called for help. Arun, a person of interest, claims he did not take the child. The case involves a missing child, potential criminal activity, and the right to life and personal liberty under Article 21 of the Indian Constitution.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = High, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 265 — Tax Not to be Imposed Save by Authority of Law**: No tax shall be levied or collected except by authority of law.
+  - Key principles: No taxation without law, Lawful authority for tax levy, Procedural fairness in tax matters
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[SECONDARY]** Article 301 — Freedom of Trade, Commerce and Intercourse**: Subject to the other provisions of this Part, trade, commerce and intercourse throughout the territory of India shall be free.
+  - Key principles: Free trade and commerce across India, No barriers to inter-state trade
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** High
+This indicates: ['Minors / Children', 'Pregnant Women', 'Elderly / Senior Citizens', 'Disabled Persons', 'Scheduled Castes (SC)', 'Scheduled Tribes (ST)', 'Other Backward Classes (OBC)', 'Adivasis / Tribals', 'Dalits', 'Economically Weaker Sections (EWS)', 'Below Poverty Line (BPL)', 'Daily Wage Workers', 'Agricultural Labourers', 'Domestic Workers', 'Migrant Workers', 'Unorganised Sector Workers', 'Bonded Labourers', 'Sex Workers', 'Human Trafficking Survivors', 'Refugees / Asylum Seekers', 'Homeless Persons', 'Orphans', 'Single Mothers / Widows', 'Persons in Custody', 'Victims of Domestic Violence', 'Victims of Sexual Assault', 'Victims of Torture']
+**Constitutional Protection:** Articles 14, 15, 15(3), 15(4), 15(5), 16(4), 17, 23, 24, 39, 39A, 41, 46, and the Directive Principles under Part IV mandate special protection for vulnerable groups. The Doctrine of Parens Patriae obligates the state to act as guardian for those who cannot protect themselves.
+**Judicial Duty:** The court must adopt a protective, sensitised approach. Vulnerable litigants are entitled to: (a) in-camera proceedings where appropriate, (b) assistance of counsel if unrepresented, (c) protection from intimidation, (d) expedited hearings to prevent secondary trauma, and (e) rehabilitation and compensation directions where applicable.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Reasonable Classification**: Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.
+  - Application to this case: Used to test whether differential treatment of litigants or groups is constitutional.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Tax and excise matters involve statutory interpretation, procedural compliance, and economic regulation. They do not typically engage the right to life under Article 21. These cases should be processed according to their legal complexity and the amount involved, but do not warrant the highest priority unless they involve personal liberty or criminal sanctions.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Party A, Party B
+**Legal Category:** Constitutional/Writ
+**Brief Description:** In this fictional scenario, Party A and Party B are involved in a violent dispute over property rights. The dispute escalated to physical harm, with Party B allegedly assaulting Party A. The case raises questions under Article 21 (right to life and personal liberty) and Article 14 (equality before law). The case falls under the Criminal/Violent category as it involves a major injury and a power imbalance.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 32 — Remedies for Enforcement of Fundamental Rights**: The right to move the Supreme Court for the enforcement of fundamental rights is guaranteed.
+  - Key principles: Right to constitutional remedies, Writ jurisdiction of Supreme Court, Enforcement of fundamental rights
+- ****[PRIMARY]** Article 226 — Power of High Courts to Issue Certain Writs**: Every High Court shall have power to issue directions, orders, or writs for enforcement of fundamental rights and for any other purpose.
+  - Key principles: Writ jurisdiction of High Courts, Judicial review of state action, Enforcement of legal rights
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[SECONDARY]** Article 227 — Power of Superintendence of High Courts**: Every High Court shall have superintendence over all courts and tribunals within its jurisdiction, and may call for returns, make rules, and settle forms to secure the proper administration of justice.
+  - Key principles: Superintendence over subordinate courts and tribunals, Administration of justice
+- ****[SECONDARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
+  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
+- ****[SECONDARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
+  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
+- ****[SECONDARY]** Article 51A — Fundamental Duties**: It shall be the duty of every citizen of India to abide by the Constitution and respect its ideals and institutions, to uphold and protect the sovereignty, unity and integrity of India, and to promote harmony and the spirit of common brotherhood.
+  - Key principles: Respect for the Constitution and its institutions, Promotion of harmony and common brotherhood, Protection of public property
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State, through the judiciary, is the ultimate guardian of fundamental rights. Under Articles 32 and 226, the High Courts and Supreme Court have a constitutional duty to protect citizens against arbitrary state action, violations of fundamental rights, and jurisdictional errors by subordinate tribunals. These cases often involve the very legitimacy of state action and require careful, principled consideration.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Basic Structure**: The Parliament cannot amend the Constitution to destroy its basic features such as supremacy of the Constitution, rule of law, and judicial review.
+  - Application to this case: Applicable to cases involving constitutional amendments or executive actions affecting foundational principles.
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+- **Doctrine of Colourable Legislation**: If the legislature lacks the competence to enact a law directly, it cannot do indirectly what it cannot do directly — such camouflage is struck down.
+  - Application to this case: Applicable where a statute purports to do one thing but in substance does another outside legislative competence.
+- **Doctrine of Harmonious Construction**: Where two constitutional provisions conflict, they should be interpreted so that both are given effect rather than one nullifying the other.
+  - Application to this case: Used when Articles or statutory provisions appear to overlap or clash.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Constitutional writ matters directly engage fundamental rights and the rule of law. Cases involving imminent threats to life or liberty (habeas corpus) warrant the highest priority. Cases challenging administrative or quasi-judicial orders should receive priority proportionate to the gravity of the rights violation alleged and the urgency of the relief sought.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
+    <t>## STATE'S CONSTITUTIONAL ASSESSMENT
+(Neutral, Unbiased Analysis from the Perspective of the Judiciary)
+This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
+### I. SUBJECT MATTER
+**Parties:** Meera Rao, Nisha Rao, Meera, Unknown Person in a Yellow Shirt, Unknown parties involved in a fictional scenario, Child, Adult, Shop Employee, Security Guard, Balloon Vendor, Suspect, Arun, Party A, Party B
+**Legal Category:** Company/Winding Up
+**Brief Description:** This case file brings together 7 documents (FIR, 6 × Other) and is assessed as a single matter of Constitutional/Writ with no injury indicated, involving vulnerable parties. The evidence on record consists of “Evidence_01_Incident_Report_and_Timeline.pdf” (FIR; Constitutional/Writ; assessed Medium priority); “Evidence_02_CCTV_Review_Log.pdf” (Other; Constitutional/Writ; assessed Medium priority); “Evidence_03_Shop_Audio_Transcript_SIMULATED.pdf” (Other; General Civil; assessed Medium priority); “Evidence_04_Witness_Statements_SIMULATED.pdf” (Other; Constitutional/Writ; assessed Medium priority); “Evidence_05_Traffic_Camera_Note.pdf” (Other; Constitutional/Writ; assessed Medium priority); “Evidence_06_Interview_Records_SIMULATED.pdf” (Other; Excise/Tax; assessed Medium priority); “Evidence_08_Evidence_Register_and_Corroboration.pdf” (Other; Constitutional/Writ; assessed Medium priority). Cross-comparison finds 4 corroborating links between the documents (shared dates, places or parties), which strengthens the consistency of the record. For example, “Evidence_01_Incident_Report_and_Timeline.pdf” and “Evidence_06_Interview_Records_SIMULATED.pdf” share parties. “Evidence_03_Shop_Audio_Transcript_SIMULATED.pdf”, “Evidence_04_Witness_Statements_SIMULATED.pdf”, “Evidence_08_Evidence_Register_and_Corroboration.pdf” currently stand alone — no other document shares a date, place or party with them, so further supporting evidence would strengthen the case.
+**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+### II. CONSTITUTIONAL RIGHTS ENGAGED
+The following constitutional provisions are relevant to this matter:
+- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+  - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
+- ****[PRIMARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
+  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
+- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
+  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
+- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[SECONDARY]** Article 39 — Certain Principles of Policy to be Followed by the State**: The State shall direct its policy towards securing equal rights to an adequate means of livelihood, and that the ownership and control of material resources are so distributed as best to subserve the common good.
+  - Key principles: Adequate means of livelihood, Distribution of material resources for common good, Prevention of concentration of wealth, Protection of workers, children and women
+- ****[SECONDARY]** Article 39A — Equal Justice and Free Legal Aid**: The State shall secure that the operation of the legal system promotes justice on a basis of equal opportunity, and shall provide free legal aid to ensure that no citizen is denied opportunities to secure justice due to economic or other disability.
+  - Key principles: Free legal aid, Equal opportunity in the legal system, Justice for the economically disadvantaged
+### III. SEVERITY &amp; URGENCY ASSESSMENT
+**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
+**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
+**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+### IV. STATE'S DUTY UNDER THE CONSTITUTION
+The State must ensure that company disputes and winding-up proceedings are adjudicated fairly, with due regard to the rights of shareholders, creditors, and employees. The judiciary must balance commercial efficiency with procedural fairness, ensuring that oppression and mismanagement claims are heard without undue delay but without displacing more urgent life-and-liberty matters.
+### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
+**Vulnerability Level:** Low
+This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
+**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
+**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Influence Level:** High
+Government bodies, large corporations, regulatory authorities, or politically powerful individuals
+**Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
+**Recommended Countermeasure:** Where there is a power imbalance, the court should: (a) ensure the weaker party has access to legal aid if needed, (b) prevent unnecessary adjournments sought by the influential party, (c) expedite proceedings to minimise the risk of witness tampering or intimidation, and (d) consider appointing a court monitor or receiver where appropriate.
+### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
+- **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
+  - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
+- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
+  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
+  - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
+### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
+**Assigned Priority:** Medium
+**Category Rationale:** Company law matters involve corporate governance, shareholder rights, and commercial disputes. While they can have significant economic consequences affecting livelihoods (Article 21), they do not involve direct threats to life or physical safety. They warrant moderated priority unless fraud, criminal conduct, or imminent liquidation threatening employee welfare is established.
+### VIII. FINAL OBSERVATION
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
+The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+  </si>
+  <si>
     <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
 **RULE 4 — Regulatory/Commercial Matter → Property &amp; Economic Rights:** Articles 14, 19(1)(g), and 300A govern this matter. Priority is based on economic impact and procedural fairness concerns, not life-and-liberty urgency.
 **FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Low**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
@@ -539,6 +1077,25 @@
 **FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Medium**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
   </si>
   <si>
+    <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
+**RULE 2 — High Vulnerability → Elevated Priority (Doctrine of Parens Patriae):** The state has a special duty to protect vulnerable persons. Articles 15, 39, and 39A require the court to ensure that vulnerable litigants are not disadvantaged by delay.
+**RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
+**RULE 4 — Constitutional/Writ Matter → Article 32/226 Jurisdiction:** The court's constitutional writ jurisdiction is engaged. Priority depends on the nature of the right sought to be enforced.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Medium**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+  </si>
+  <si>
+    <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
+**RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Medium**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+  </si>
+  <si>
+    <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
+**RULE 2 — High Vulnerability → Elevated Priority (Doctrine of Parens Patriae):** The state has a special duty to protect vulnerable persons. Articles 15, 39, and 39A require the court to ensure that vulnerable litigants are not disadvantaged by delay.
+**RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
+**RULE 4 — Regulatory/Commercial Matter → Property &amp; Economic Rights:** Articles 14, 19(1)(g), and 300A govern this matter. Priority is based on economic impact and procedural fairness concerns, not life-and-liberty urgency.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Medium**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+  </si>
+  <si>
     <t>case_priority_system\decision_graphs\03_Exhibit_P2_Bank_Transfers_decision_report.md</t>
   </si>
   <si>
@@ -560,6 +1117,30 @@
     <t>case_priority_system/decision_graphs\ANV-2026-0019_whole_case_decision_report.md</t>
   </si>
   <si>
+    <t>case_priority_system/decision_graphs\Evidence_01_Incident_Report_and_Timeline_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Evidence_02_CCTV_Review_Log_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Evidence_03_Shop_Audio_Transcript_SIMULATED_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Evidence_04_Witness_Statements_SIMULATED_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Evidence_05_Traffic_Camera_Note_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Evidence_06_Interview_Records_SIMULATED_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\Evidence_08_Evidence_Register_and_Corroboration_decision_report.md</t>
+  </si>
+  <si>
+    <t>case_priority_system/decision_graphs\ANV-2026-0025_whole_case_decision_report.md</t>
+  </si>
+  <si>
     <t>Low</t>
   </si>
   <si>
@@ -575,6 +1156,9 @@
     <t>Constitutional/Writ</t>
   </si>
   <si>
+    <t>Company/Winding Up</t>
+  </si>
+  <si>
     <t>Non-Violent</t>
   </si>
   <si>
@@ -596,7 +1180,28 @@
     <t>[{'article': 'Article 32', 'title': 'Remedies for Enforcement of Fundamental Rights', 'primary': True, 'why_applies': 'This case has been filed directly in the Supreme Court. Article 32 gives every citizen the right to go to the Supreme Court if their basic rights are being taken away. It is the tool that makes sure all the other rights actually work.', 'precedents': []}, {'article': 'Article 226', 'title': 'Power of High Courts to Issue Certain Writs', 'primary': True, 'why_applies': 'This case has been filed in a High Court. Article 226 gives High Courts the power to order the government to follow the law. If a government body does something illegal, this article lets citizens ask the court to step in and fix it.', 'precedents': []}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other. One side is much more powerful than the other — a government body, a large company, or someone with political influence. Article 14 requires the court to make sure the weaker party is not overpowered.', 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason.", 'precedents': []}, {'article': 'Article 227', 'title': 'Power of Superintendence of High Courts', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 22', 'title': 'Protection Against Arrest and Detention', 'primary': False, 'why_applies': 'Someone has been arrested. Article 22 says they must be told why, allowed to talk to a lawyer, and not kept in jail forever without a proper hearing. It protects people from being locked up without reason.', 'precedents': []}, {'article': 'Article 20', 'title': 'Protection in Respect of Conviction for Offences', 'primary': False, 'why_applies': 'This is a criminal case. Article 20 protects the accused person from being treated unfairly. It says: you cannot be punished for something that was not a crime when you did it, you cannot be tried twice for the same offence, and you cannot be forced to confess.', 'precedents': []}, {'article': 'Article 51A', 'title': 'Fundamental Duties', 'primary': False, 'why_applies': '', 'precedents': []}]</t>
   </si>
   <si>
+    <t>[{'article': 'Article 32', 'title': 'Remedies for Enforcement of Fundamental Rights', 'primary': True, 'why_applies': 'This case has been filed directly in the Supreme Court. Article 32 gives every citizen the right to go to the Supreme Court if their basic rights are being taken away. It is the tool that makes sure all the other rights actually work.', 'precedents': []}, {'article': 'Article 226', 'title': 'Power of High Courts to Issue Certain Writs', 'primary': True, 'why_applies': 'This case has been filed in a High Court. Article 226 gives High Courts the power to order the government to follow the law. If a government body does something illegal, this article lets citizens ask the court to step in and fix it.', 'precedents': []}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other. A vulnerable person is involved — like a child, an elderly person, or someone from a disadvantaged community. The government has a special duty to protect them. One side is much more powerful than the other — a government body, a large company, or someone with political influence. Article 14 requires the court to make sure the weaker party is not overpowered.', 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason. A vulnerable person is involved — like a child, an elderly person, or someone from a disadvantaged community. The government has a special duty to protect them.", 'precedents': []}, {'article': 'Article 227', 'title': 'Power of Superintendence of High Courts', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 22', 'title': 'Protection Against Arrest and Detention', 'primary': False, 'why_applies': 'Someone has been arrested. Article 22 says they must be told why, allowed to talk to a lawyer, and not kept in jail forever without a proper hearing. It protects people from being locked up without reason.', 'precedents': []}, {'article': 'Article 20', 'title': 'Protection in Respect of Conviction for Offences', 'primary': False, 'why_applies': 'This is a criminal case. Article 20 protects the accused person from being treated unfairly. It says: you cannot be punished for something that was not a crime when you did it, you cannot be tried twice for the same offence, and you cannot be forced to confess.', 'precedents': []}, {'article': 'Article 51A', 'title': 'Fundamental Duties', 'primary': False, 'why_applies': '', 'precedents': []}]</t>
+  </si>
+  <si>
+    <t>[{'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other. One side is much more powerful than the other — a government body, a large company, or someone with political influence. Article 14 requires the court to make sure the weaker party is not overpowered.', 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason.", 'precedents': []}, {'article': 'Article 39A', 'title': 'Equal Justice and Free Legal Aid', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 44', 'title': 'Uniform Civil Code', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 51A', 'title': 'Fundamental Duties', 'primary': False, 'why_applies': '', 'precedents': []}]</t>
+  </si>
+  <si>
+    <t>[{'article': 'Article 265', 'title': 'Tax Not to be Imposed Save by Authority of Law', 'primary': True, 'why_applies': 'This is a tax case. Article 265 says the government cannot collect any tax unless a law specifically allows it. If the tax was charged without proper legal backing, it must be given back.', 'precedents': []}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other. A vulnerable person is involved — like a child, an elderly person, or someone from a disadvantaged community. The government has a special duty to protect them. One side is much more powerful than the other — a government body, a large company, or someone with political influence. Article 14 requires the court to make sure the weaker party is not overpowered.', 'precedents': []}, {'article': 'Article 19(1)(g)', 'title': 'Right to Practise Any Profession or Carry On Occupation, Trade or Business', 'primary': True, 'why_applies': "This case is about someone's right to run a business, practice a trade, or do a job. Article 19(1)(g) protects that right, but the government can put fair limits on it if the public interest requires it. The court must decide if those limits were reasonable.", 'precedents': []}, {'article': 'Article 300A', 'title': 'Right to Property', 'primary': False, 'why_applies': 'This case involves property or money. Article 300A protects people from losing their property without a lawful reason. The court must check that the proper legal process was followed.', 'precedents': []}, {'article': 'Article 301', 'title': 'Freedom of Trade, Commerce and Intercourse', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': False, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason. A vulnerable person is involved — like a child, an elderly person, or someone from a disadvantaged community. The government has a special duty to protect them.", 'precedents': []}]</t>
+  </si>
+  <si>
+    <t>[{'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other. One side is much more powerful than the other — a government body, a large company, or someone with political influence. Article 14 requires the court to make sure the weaker party is not overpowered.', 'precedents': []}, {'article': 'Article 300A', 'title': 'Right to Property', 'primary': True, 'why_applies': 'This case involves property or money. Article 300A protects people from losing their property without a lawful reason. The court must check that the proper legal process was followed.', 'precedents': []}, {'article': 'Article 19(1)(g)', 'title': 'Right to Practise Any Profession or Carry On Occupation, Trade or Business', 'primary': True, 'why_applies': "This case is about someone's right to run a business, practice a trade, or do a job. Article 19(1)(g) protects that right, but the government can put fair limits on it if the public interest requires it. The court must decide if those limits were reasonable.", 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': False, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason.", 'precedents': []}, {'article': 'Article 39', 'title': 'Certain Principles of Policy to be Followed by the State', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 39A', 'title': 'Equal Justice and Free Legal Aid', 'primary': False, 'why_applies': '', 'precedents': []}]</t>
+  </si>
+  <si>
     <t>Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.</t>
+  </si>
+  <si>
+    <t>The State, through the judiciary, is the ultimate guardian of fundamental rights. Under Articles 32 and 226, the High Courts and Supreme Court have a constitutional duty to protect citizens against arbitrary state action, violations of fundamental rights, and jurisdictional errors by subordinate tribunals. These cases often involve the very legitimacy of state action and require careful, principled consideration.</t>
+  </si>
+  <si>
+    <t>The State must ensure that all civil disputes are adjudicated fairly, transparently, and within a reasonable time. Under Article 14, the state guarantees equal access to justice — all litigants are entitled to a fair hearing. The principle of speedy trial (derived from Article 21) requires that even ordinary civil matters be resolved without inordinate delay, though they yield priority to cases involving life and liberty.</t>
+  </si>
+  <si>
+    <t>The State must ensure that company disputes and winding-up proceedings are adjudicated fairly, with due regard to the rights of shareholders, creditors, and employees. The judiciary must balance commercial efficiency with procedural fairness, ensuring that oppression and mismanagement claims are heard without undue delay but without displacing more urgent life-and-liberty matters.</t>
   </si>
   <si>
     <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}, {'name': 'Doctrine of Reasonable Classification', 'description': 'Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.', 'application': 'Used to test whether differential treatment of litigants or groups is constitutional.'}]</t>
@@ -625,6 +1230,27 @@
 **Category-Specific Analysis — Constitutional/Writ:** Writ matters directly engage the court's constitutional jurisdiction under Articles 32 and 226. The priority should reflect the nature of the right sought to be enforced — habeas corpus (life/liberty) cases require the highest priority.</t>
   </si>
   <si>
+    <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Vulnerability Analysis — Special State Obligation:** A vulnerable party is involved. The Doctrine of Parens Patriae and Articles 15(3), 15(4), 39, and 39A impose a heightened duty on the state to protect the vulnerable. This factor strongly supports elevated priority to prevent further harm or injustice.
+**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
+**Category-Specific Analysis — Constitutional/Writ:** Writ matters directly engage the court's constitutional jurisdiction under Articles 32 and 226. The priority should reflect the nature of the right sought to be enforced — habeas corpus (life/liberty) cases require the highest priority.</t>
+  </si>
+  <si>
+    <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.</t>
+  </si>
+  <si>
+    <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Vulnerability Analysis — Special State Obligation:** A vulnerable party is involved. The Doctrine of Parens Patriae and Articles 15(3), 15(4), 39, and 39A impose a heightened duty on the state to protect the vulnerable. This factor strongly supports elevated priority to prevent further harm or injustice.
+**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
+**Category-Specific Analysis — Excise/Tax:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
+  </si>
+  <si>
+    <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+**Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
+**Category-Specific Analysis — Company/Winding Up:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
+  </si>
+  <si>
     <t>case_priority_system\reports\03_Exhibit_P2_Bank_Transfers_report.pdf</t>
   </si>
   <si>
@@ -646,13 +1272,43 @@
     <t>case_priority_system/reports\ANV-2026-0019_whole_case_report.pdf</t>
   </si>
   <si>
+    <t>case_priority_system\reports\Evidence_01_Incident_Report_and_Timeline_report.pdf</t>
+  </si>
+  <si>
+    <t>case_priority_system\reports\Evidence_02_CCTV_Review_Log_report.pdf</t>
+  </si>
+  <si>
+    <t>case_priority_system\reports\Evidence_03_Shop_Audio_Transcript_SIMULATED_report.pdf</t>
+  </si>
+  <si>
+    <t>case_priority_system\reports\Evidence_04_Witness_Statements_SIMULATED_report.pdf</t>
+  </si>
+  <si>
+    <t>case_priority_system\reports\Evidence_05_Traffic_Camera_Note_report.pdf</t>
+  </si>
+  <si>
+    <t>case_priority_system\reports\Evidence_06_Interview_Records_SIMULATED_report.pdf</t>
+  </si>
+  <si>
+    <t>case_priority_system\reports\Evidence_08_Evidence_Register_and_Corroboration_report.pdf</t>
+  </si>
+  <si>
+    <t>case_priority_system/reports\ANV-2026-0025_whole_case_report.pdf</t>
+  </si>
+  <si>
     <t>ANV-2026-0019</t>
   </si>
   <si>
+    <t>ANV-2026-0025</t>
+  </si>
+  <si>
     <t>Other</t>
   </si>
   <si>
     <t>Whole Case</t>
+  </si>
+  <si>
+    <t>FIR</t>
   </si>
 </sst>
 </file>
@@ -984,7 +1640,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1054,58 +1710,58 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="F2" t="s">
-        <v>51</v>
+        <v>86</v>
       </c>
       <c r="G2" t="s">
-        <v>51</v>
+        <v>86</v>
       </c>
       <c r="H2" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="I2" t="s">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="J2" t="s">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="K2" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="L2" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="M2" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="N2" t="s">
-        <v>66</v>
+        <v>110</v>
       </c>
       <c r="P2" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="Q2" t="s">
-        <v>74</v>
+        <v>125</v>
       </c>
       <c r="R2" t="s">
-        <v>78</v>
+        <v>133</v>
       </c>
       <c r="S2" t="s">
-        <v>85</v>
+        <v>148</v>
       </c>
       <c r="T2" t="s">
-        <v>86</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1113,58 +1769,58 @@
         <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="F3" t="s">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="G3" t="s">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="H3" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="I3" t="s">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="J3" t="s">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="K3" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="L3" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="M3" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="N3" t="s">
-        <v>66</v>
+        <v>110</v>
       </c>
       <c r="P3" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="Q3" t="s">
-        <v>74</v>
+        <v>125</v>
       </c>
       <c r="R3" t="s">
-        <v>79</v>
+        <v>134</v>
       </c>
       <c r="S3" t="s">
-        <v>85</v>
+        <v>148</v>
       </c>
       <c r="T3" t="s">
-        <v>86</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1172,58 +1828,58 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>53</v>
+        <v>88</v>
       </c>
       <c r="G4" t="s">
-        <v>53</v>
+        <v>88</v>
       </c>
       <c r="H4" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="I4" t="s">
-        <v>61</v>
+        <v>104</v>
       </c>
       <c r="J4" t="s">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="K4" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="L4" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="M4" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="N4" t="s">
-        <v>67</v>
+        <v>111</v>
       </c>
       <c r="P4" t="s">
-        <v>72</v>
+        <v>123</v>
       </c>
       <c r="Q4" t="s">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="R4" t="s">
-        <v>80</v>
+        <v>135</v>
       </c>
       <c r="S4" t="s">
-        <v>85</v>
+        <v>148</v>
       </c>
       <c r="T4" t="s">
-        <v>86</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1231,58 +1887,58 @@
         <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="E5" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
       <c r="F5" t="s">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="H5" t="s">
-        <v>59</v>
+        <v>102</v>
       </c>
       <c r="I5" t="s">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="J5" t="s">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="K5" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="L5" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="M5" t="s">
-        <v>65</v>
+        <v>109</v>
       </c>
       <c r="N5" t="s">
-        <v>68</v>
+        <v>112</v>
       </c>
       <c r="P5" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="Q5" t="s">
-        <v>76</v>
+        <v>127</v>
       </c>
       <c r="R5" t="s">
-        <v>81</v>
+        <v>136</v>
       </c>
       <c r="S5" t="s">
-        <v>85</v>
+        <v>148</v>
       </c>
       <c r="T5" t="s">
-        <v>86</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -1290,58 +1946,58 @@
         <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="E6" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="F6" t="s">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="G6" t="s">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="H6" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="I6" t="s">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="J6" t="s">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="K6" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="L6" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="M6" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="N6" t="s">
-        <v>66</v>
+        <v>110</v>
       </c>
       <c r="P6" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="Q6" t="s">
-        <v>74</v>
+        <v>125</v>
       </c>
       <c r="R6" t="s">
-        <v>82</v>
+        <v>137</v>
       </c>
       <c r="S6" t="s">
-        <v>85</v>
+        <v>148</v>
       </c>
       <c r="T6" t="s">
-        <v>86</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -1349,58 +2005,58 @@
         <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="F7" t="s">
-        <v>56</v>
+        <v>91</v>
       </c>
       <c r="G7" t="s">
-        <v>56</v>
+        <v>91</v>
       </c>
       <c r="H7" t="s">
-        <v>59</v>
+        <v>102</v>
       </c>
       <c r="I7" t="s">
-        <v>62</v>
+        <v>105</v>
       </c>
       <c r="J7" t="s">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="K7" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="L7" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="M7" t="s">
-        <v>65</v>
+        <v>109</v>
       </c>
       <c r="N7" t="s">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="P7" t="s">
-        <v>73</v>
+        <v>124</v>
       </c>
       <c r="Q7" t="s">
-        <v>77</v>
+        <v>128</v>
       </c>
       <c r="R7" t="s">
-        <v>83</v>
+        <v>138</v>
       </c>
       <c r="S7" t="s">
-        <v>85</v>
+        <v>148</v>
       </c>
       <c r="T7" t="s">
-        <v>86</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -1408,61 +2064,557 @@
         <v>26</v>
       </c>
       <c r="B8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" t="s">
+        <v>81</v>
+      </c>
+      <c r="F8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H8" t="s">
+        <v>102</v>
+      </c>
+      <c r="I8" t="s">
+        <v>103</v>
+      </c>
+      <c r="J8" t="s">
+        <v>107</v>
+      </c>
+      <c r="K8" t="s">
+        <v>108</v>
+      </c>
+      <c r="L8" t="s">
+        <v>101</v>
+      </c>
+      <c r="M8" t="s">
+        <v>109</v>
+      </c>
+      <c r="N8" t="s">
+        <v>112</v>
+      </c>
+      <c r="O8" t="s">
+        <v>118</v>
+      </c>
+      <c r="P8" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>127</v>
+      </c>
+      <c r="R8" t="s">
+        <v>139</v>
+      </c>
+      <c r="S8" t="s">
+        <v>148</v>
+      </c>
+      <c r="T8" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" t="s">
+        <v>93</v>
+      </c>
+      <c r="G9" t="s">
+        <v>93</v>
+      </c>
+      <c r="H9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I9" t="s">
+        <v>105</v>
+      </c>
+      <c r="J9" t="s">
+        <v>107</v>
+      </c>
+      <c r="K9" t="s">
+        <v>108</v>
+      </c>
+      <c r="L9" t="s">
+        <v>109</v>
+      </c>
+      <c r="M9" t="s">
+        <v>109</v>
+      </c>
+      <c r="N9" t="s">
+        <v>114</v>
+      </c>
+      <c r="O9" t="s">
+        <v>119</v>
+      </c>
+      <c r="P9" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>129</v>
+      </c>
+      <c r="R9" t="s">
+        <v>140</v>
+      </c>
+      <c r="S9" t="s">
+        <v>149</v>
+      </c>
+      <c r="T9" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20">
+      <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10" t="s">
+        <v>94</v>
+      </c>
+      <c r="G10" t="s">
+        <v>94</v>
+      </c>
+      <c r="H10" t="s">
+        <v>102</v>
+      </c>
+      <c r="I10" t="s">
+        <v>105</v>
+      </c>
+      <c r="J10" t="s">
+        <v>107</v>
+      </c>
+      <c r="K10" t="s">
+        <v>108</v>
+      </c>
+      <c r="L10" t="s">
+        <v>101</v>
+      </c>
+      <c r="M10" t="s">
+        <v>109</v>
+      </c>
+      <c r="N10" t="s">
+        <v>113</v>
+      </c>
+      <c r="O10" t="s">
+        <v>119</v>
+      </c>
+      <c r="P10" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>128</v>
+      </c>
+      <c r="R10" t="s">
+        <v>141</v>
+      </c>
+      <c r="S10" t="s">
+        <v>149</v>
+      </c>
+      <c r="T10" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20">
+      <c r="A11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G11" t="s">
+        <v>95</v>
+      </c>
+      <c r="H11" t="s">
+        <v>102</v>
+      </c>
+      <c r="I11" t="s">
+        <v>104</v>
+      </c>
+      <c r="J11" t="s">
+        <v>107</v>
+      </c>
+      <c r="K11" t="s">
+        <v>108</v>
+      </c>
+      <c r="L11" t="s">
+        <v>101</v>
+      </c>
+      <c r="M11" t="s">
+        <v>109</v>
+      </c>
+      <c r="N11" t="s">
+        <v>115</v>
+      </c>
+      <c r="O11" t="s">
+        <v>120</v>
+      </c>
+      <c r="P11" t="s">
+        <v>123</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>130</v>
+      </c>
+      <c r="R11" t="s">
+        <v>142</v>
+      </c>
+      <c r="S11" t="s">
+        <v>149</v>
+      </c>
+      <c r="T11" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" t="s">
+        <v>96</v>
+      </c>
+      <c r="G12" t="s">
+        <v>96</v>
+      </c>
+      <c r="H12" t="s">
+        <v>102</v>
+      </c>
+      <c r="I12" t="s">
+        <v>105</v>
+      </c>
+      <c r="J12" t="s">
+        <v>107</v>
+      </c>
+      <c r="K12" t="s">
+        <v>108</v>
+      </c>
+      <c r="L12" t="s">
+        <v>109</v>
+      </c>
+      <c r="M12" t="s">
+        <v>109</v>
+      </c>
+      <c r="N12" t="s">
+        <v>114</v>
+      </c>
+      <c r="O12" t="s">
+        <v>119</v>
+      </c>
+      <c r="P12" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>129</v>
+      </c>
+      <c r="R12" t="s">
+        <v>143</v>
+      </c>
+      <c r="S12" t="s">
+        <v>149</v>
+      </c>
+      <c r="T12" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" t="s">
+        <v>82</v>
+      </c>
+      <c r="F13" t="s">
+        <v>97</v>
+      </c>
+      <c r="G13" t="s">
+        <v>97</v>
+      </c>
+      <c r="H13" t="s">
+        <v>102</v>
+      </c>
+      <c r="I13" t="s">
+        <v>105</v>
+      </c>
+      <c r="J13" t="s">
+        <v>107</v>
+      </c>
+      <c r="K13" t="s">
+        <v>108</v>
+      </c>
+      <c r="L13" t="s">
+        <v>101</v>
+      </c>
+      <c r="M13" t="s">
+        <v>109</v>
+      </c>
+      <c r="N13" t="s">
+        <v>113</v>
+      </c>
+      <c r="O13" t="s">
+        <v>119</v>
+      </c>
+      <c r="P13" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>128</v>
+      </c>
+      <c r="R13" t="s">
+        <v>144</v>
+      </c>
+      <c r="S13" t="s">
+        <v>149</v>
+      </c>
+      <c r="T13" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20">
+      <c r="A14" t="s">
         <v>32</v>
       </c>
-      <c r="C8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="B14" t="s">
         <v>46</v>
       </c>
-      <c r="E8" t="s">
-        <v>49</v>
-      </c>
-      <c r="F8" t="s">
-        <v>57</v>
-      </c>
-      <c r="G8" t="s">
-        <v>57</v>
-      </c>
-      <c r="H8" t="s">
-        <v>59</v>
-      </c>
-      <c r="I8" t="s">
-        <v>60</v>
-      </c>
-      <c r="J8" t="s">
+      <c r="C14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" t="s">
+        <v>98</v>
+      </c>
+      <c r="G14" t="s">
+        <v>98</v>
+      </c>
+      <c r="H14" t="s">
+        <v>102</v>
+      </c>
+      <c r="I14" t="s">
+        <v>103</v>
+      </c>
+      <c r="J14" t="s">
+        <v>107</v>
+      </c>
+      <c r="K14" t="s">
+        <v>108</v>
+      </c>
+      <c r="L14" t="s">
+        <v>109</v>
+      </c>
+      <c r="M14" t="s">
+        <v>109</v>
+      </c>
+      <c r="N14" t="s">
+        <v>116</v>
+      </c>
+      <c r="O14" t="s">
+        <v>118</v>
+      </c>
+      <c r="P14" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>131</v>
+      </c>
+      <c r="R14" t="s">
+        <v>145</v>
+      </c>
+      <c r="S14" t="s">
+        <v>149</v>
+      </c>
+      <c r="T14" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D15" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" t="s">
+        <v>82</v>
+      </c>
+      <c r="F15" t="s">
+        <v>99</v>
+      </c>
+      <c r="G15" t="s">
+        <v>99</v>
+      </c>
+      <c r="H15" t="s">
+        <v>102</v>
+      </c>
+      <c r="I15" t="s">
+        <v>105</v>
+      </c>
+      <c r="J15" t="s">
+        <v>107</v>
+      </c>
+      <c r="K15" t="s">
+        <v>108</v>
+      </c>
+      <c r="L15" t="s">
+        <v>101</v>
+      </c>
+      <c r="M15" t="s">
+        <v>109</v>
+      </c>
+      <c r="N15" t="s">
+        <v>113</v>
+      </c>
+      <c r="O15" t="s">
+        <v>119</v>
+      </c>
+      <c r="P15" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>128</v>
+      </c>
+      <c r="R15" t="s">
+        <v>146</v>
+      </c>
+      <c r="S15" t="s">
+        <v>149</v>
+      </c>
+      <c r="T15" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20">
+      <c r="A16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" t="s">
         <v>63</v>
       </c>
-      <c r="K8" t="s">
-        <v>64</v>
-      </c>
-      <c r="L8" t="s">
-        <v>58</v>
-      </c>
-      <c r="M8" t="s">
-        <v>65</v>
-      </c>
-      <c r="N8" t="s">
-        <v>68</v>
-      </c>
-      <c r="O8" t="s">
-        <v>70</v>
-      </c>
-      <c r="P8" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>76</v>
-      </c>
-      <c r="R8" t="s">
-        <v>84</v>
-      </c>
-      <c r="S8" t="s">
-        <v>85</v>
-      </c>
-      <c r="T8" t="s">
-        <v>87</v>
+      <c r="D16" t="s">
+        <v>78</v>
+      </c>
+      <c r="E16" t="s">
+        <v>81</v>
+      </c>
+      <c r="F16" t="s">
+        <v>100</v>
+      </c>
+      <c r="G16" t="s">
+        <v>100</v>
+      </c>
+      <c r="H16" t="s">
+        <v>102</v>
+      </c>
+      <c r="I16" t="s">
+        <v>106</v>
+      </c>
+      <c r="J16" t="s">
+        <v>107</v>
+      </c>
+      <c r="K16" t="s">
+        <v>108</v>
+      </c>
+      <c r="L16" t="s">
+        <v>101</v>
+      </c>
+      <c r="M16" t="s">
+        <v>109</v>
+      </c>
+      <c r="N16" t="s">
+        <v>117</v>
+      </c>
+      <c r="O16" t="s">
+        <v>121</v>
+      </c>
+      <c r="P16" t="s">
+        <v>123</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>132</v>
+      </c>
+      <c r="R16" t="s">
+        <v>147</v>
+      </c>
+      <c r="S16" t="s">
+        <v>149</v>
+      </c>
+      <c r="T16" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(docket): synchronize ANV-2026-0025 whole-case priority to High in case_results.xlsx
</commit_message>
<xml_diff>
--- a/case_priority_system/case_results.xlsx
+++ b/case_priority_system/case_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="157">
   <si>
     <t>Case_File</t>
   </si>
@@ -1009,34 +1009,38 @@
 This assessment is prepared from the standpoint of an impartial state adjudicating disputes under the Constitution of India. The analysis identifies the constitutional rights engaged, the state's corresponding duties, and the appropriate priority that a fair and unbiased judiciary should accord to this matter.
 ### I. SUBJECT MATTER
 **Parties:** Meera Rao, Nisha Rao, Meera, Unknown Person in a Yellow Shirt, Unknown parties involved in a fictional scenario, Child, Adult, Shop Employee, Security Guard, Balloon Vendor, Suspect, Arun, Party A, Party B
-**Legal Category:** Company/Winding Up
+**Legal Category:** Criminal/Violent
 **Brief Description:** This case file brings together 7 documents (FIR, 6 × Other) and is assessed as a single matter of Constitutional/Writ with no injury indicated, involving vulnerable parties. The evidence on record consists of “Evidence_01_Incident_Report_and_Timeline.pdf” (FIR; Constitutional/Writ; assessed Medium priority); “Evidence_02_CCTV_Review_Log.pdf” (Other; Constitutional/Writ; assessed Medium priority); “Evidence_03_Shop_Audio_Transcript_SIMULATED.pdf” (Other; General Civil; assessed Medium priority); “Evidence_04_Witness_Statements_SIMULATED.pdf” (Other; Constitutional/Writ; assessed Medium priority); “Evidence_05_Traffic_Camera_Note.pdf” (Other; Constitutional/Writ; assessed Medium priority); “Evidence_06_Interview_Records_SIMULATED.pdf” (Other; Excise/Tax; assessed Medium priority); “Evidence_08_Evidence_Register_and_Corroboration.pdf” (Other; Constitutional/Writ; assessed Medium priority). Cross-comparison finds 4 corroborating links between the documents (shared dates, places or parties), which strengthens the consistency of the record. For example, “Evidence_01_Incident_Report_and_Timeline.pdf” and “Evidence_06_Interview_Records_SIMULATED.pdf” share parties. “Evidence_03_Shop_Audio_Transcript_SIMULATED.pdf”, “Evidence_04_Witness_Statements_SIMULATED.pdf”, “Evidence_08_Evidence_Register_and_Corroboration.pdf” currently stand alone — no other document shares a date, place or party with them, so further supporting evidence would strengthen the case.
-**Extracted Parameters:** Severity = No Injury, Vulnerability = Low, Influence/ Power Imbalance = High
+**Extracted Parameters:** Severity = Major, Vulnerability = High, Influence/ Power Imbalance = High
 ### II. CONSTITUTIONAL RIGHTS ENGAGED
 The following constitutional provisions are relevant to this matter:
-- ****[PRIMARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
+- ****[PRIMARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
+  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
+- ****[PRIMARY]** Article 22 — Protection Against Arrest and Detention**: No person who is arrested shall be detained in custody without being informed of the grounds of arrest, nor shall he be denied the right to consult and be defended by a legal practitioner of his choice. Every person detained under preventive detention must be informed of the grounds of detention.
+  - Key principles: Right to be informed of grounds of arrest, Right to consult a lawyer, Safeguards against arbitrary detention, Preventive detention procedural safeguards
+- ****[PRIMARY]** Article 20 — Protection in Respect of Conviction for Offences**: No person shall be convicted of any offence except for violation of a law in force at the time of the act. No person shall be prosecuted and punished for the same offence more than once. No person accused of any offence shall be compelled to be a witness against himself.
+  - Key principles: No ex post facto criminal law, No double jeopardy, Protection against self-incrimination
+- ****[SECONDARY]** Article 14 — Equality Before Law**: The State shall not deny to any person equality before the law or the equal protection of the laws within the territory of India.
   - Key principles: Equality before law, Equal protection of laws, Reasonable classification is permitted, Anti-arbitrariness
-- ****[PRIMARY]** Article 300A — Right to Property**: No person shall be deprived of his property save by authority of law.
-  - Key principles: Protection against deprivation of property, Lawful procedure for acquisition, Right not to be dispossessed without legal authority
-- ****[PRIMARY]** Article 19(1)(g) — Right to Practise Any Profession or Carry On Occupation, Trade or Business**: All citizens shall have the right to practise any profession, or to carry on any occupation, trade or business, subject to reasonable restrictions in the interests of the general public.
-  - Key principles: Right to trade, occupation and profession, Reasonable restrictions in public interest, Licensing and regulatory controls
-- ****[SECONDARY]** Article 21 — Protection of Life and Personal Liberty**: No person shall be deprived of his life or personal liberty except according to procedure established by law.
-  - Key principles: Right to life includes right to live with dignity, Right to a speedy trial, Right to health and medical care, Right to fair procedure, Right to safety and security, Due process and procedural fairness
-- ****[SECONDARY]** Article 39 — Certain Principles of Policy to be Followed by the State**: The State shall direct its policy towards securing equal rights to an adequate means of livelihood, and that the ownership and control of material resources are so distributed as best to subserve the common good.
-  - Key principles: Adequate means of livelihood, Distribution of material resources for common good, Prevention of concentration of wealth, Protection of workers, children and women
+- ****[SECONDARY]** Article 17 — Abolition of Untouchability**: Untouchability is abolished and its practice in any form is forbidden. The enforcement of any disability arising out of untouchability shall be an offence punishable in accordance with law.
+  - Key principles: Abolition of untouchability, Enforcement of disabilities is an offence, Protection of SC/ST communities
+- ****[SECONDARY]** Article 23 — Prohibition of Traffic in Human Beings and Forced Labour**: Traffic in human beings and begar and other similar forms of forced labour are prohibited. Any contravention of this provision shall be an offence punishable in accordance with law.
+  - Key principles: Prohibition of human trafficking, Prohibition of forced labour and begar
+- ****[SECONDARY]** Article 24 — Prohibition of Employment of Children in Factories**: No child below the age of fourteen years shall be employed to work in any factory or mine or engaged in any other hazardous employment.
+  - Key principles: No child labour below 14 in hazardous work, Protection of children from exploitation
 - ****[SECONDARY]** Article 39A — Equal Justice and Free Legal Aid**: The State shall secure that the operation of the legal system promotes justice on a basis of equal opportunity, and shall provide free legal aid to ensure that no citizen is denied opportunities to secure justice due to economic or other disability.
   - Key principles: Free legal aid, Equal opportunity in the legal system, Justice for the economically disadvantaged
 ### III. SEVERITY &amp; URGENCY ASSESSMENT
-**Primary Article:** Article 14 / Article 19 / Article 300A (as applicable)
-**Analysis:** Where no physical injury is involved, the primary constitutional concern shifts from Article 21 (life and liberty) to other guarantees such as Article 14 (equality), Article 19 (freedom of profession/trade), and Article 300A (property). While these rights are fundamental and must be protected, the urgency is generally lower than cases involving threats to life or physical safety.
-**Urgency Classification:** Standard — rights are engaged but no immediate physical harm.
+**Primary Article:** Article 21
+**Analysis:** The right to life under Article 21 includes the right to live with dignity and the right to health. Major injuries — especially those requiring hospitalisation, causing permanent disability, or posing life-threatening complications — constitute a serious interference with personal liberty and bodily integrity. The State must ensure prompt access to medical care, investigation of the incident, and accountability. Each day of delay risks permanent aggravation of the harm.
+**Urgency Classification:** High — bodily integrity and dignity are seriously compromised.
 ### IV. STATE'S DUTY UNDER THE CONSTITUTION
-The State must ensure that company disputes and winding-up proceedings are adjudicated fairly, with due regard to the rights of shareholders, creditors, and employees. The judiciary must balance commercial efficiency with procedural fairness, ensuring that oppression and mismanagement claims are heard without undue delay but without displacing more urgent life-and-liberty matters.
+The State has a non-derogable duty under Article 21 to protect the right to life and personal liberty of every person. In violent crimes, the judiciary must ensure: (a) immediate protection of the victim and witnesses, (b) preservation of evidence, (c) expeditious trial to prevent secondary victimisation, and (d) enforcement of the victim's right to a speedy trial as an integral part of Article 21.
 ### V. VULNERABILITY &amp; POWER BALANCE ASSESSMENT
-**Vulnerability Level:** Low
-This indicates: ['Corporate entities', 'Well-established businesses', 'Government bodies', 'Public sector undertakings', 'High net-worth individuals', 'Professional litigants']
-**Constitutional Protection:** Article 14 guarantees equal protection of laws. These parties are expected to have access to legal representation and the ability to present their case effectively.
-**Judicial Duty:** Standard procedural fairness applies. No special accommodation beyond ordinary courtesies is required.
+**Vulnerability Level:** High
+This indicates: ['Minors / Children', 'Pregnant Women', 'Elderly / Senior Citizens', 'Disabled Persons', 'Scheduled Castes (SC)', 'Scheduled Tribes (ST)', 'Other Backward Classes (OBC)', 'Adivasis / Tribals', 'Dalits', 'Economically Weaker Sections (EWS)', 'Below Poverty Line (BPL)', 'Daily Wage Workers', 'Agricultural Labourers', 'Domestic Workers', 'Migrant Workers', 'Unorganised Sector Workers', 'Bonded Labourers', 'Sex Workers', 'Human Trafficking Survivors', 'Refugees / Asylum Seekers', 'Homeless Persons', 'Orphans', 'Single Mothers / Widows', 'Persons in Custody', 'Victims of Domestic Violence', 'Victims of Sexual Assault', 'Victims of Torture']
+**Constitutional Protection:** Articles 14, 15, 15(3), 15(4), 15(5), 16(4), 17, 23, 24, 39, 39A, 41, 46, and the Directive Principles under Part IV mandate special protection for vulnerable groups. The Doctrine of Parens Patriae obligates the state to act as guardian for those who cannot protect themselves.
+**Judicial Duty:** The court must adopt a protective, sensitised approach. Vulnerable litigants are entitled to: (a) in-camera proceedings where appropriate, (b) assistance of counsel if unrepresented, (c) protection from intimidation, (d) expedited hearings to prevent secondary trauma, and (e) rehabilitation and compensation directions where applicable.
 **Influence Level:** High
 Government bodies, large corporations, regulatory authorities, or politically powerful individuals
 **Constitutional Concern:** Article 14 requires equality before law. A significant power imbalance can undermine the fairness of proceedings if the influential party is able to use its resources to delay, intimidate, or out-litigate the weaker party. The court must actively ensure a level playing field.
@@ -1044,16 +1048,16 @@
 ### VI. APPLICABLE CONSTITUTIONAL DOCTRINES &amp; PRINCIPLES
 - **Doctrine of Proportionality**: Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.
   - Application to this case: Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.
-- **Principle of Natural Justice — Audi Alteram Partem**: No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.
-  - Application to this case: Ensures procedural fairness in administrative and quasi-judicial proceedings.
+- **Doctrine of Parens Patriae**: The state has a duty to protect those who cannot protect themselves, such as minors, disabled persons, and the mentally ill.
+  - Application to this case: Critical for cases involving vulnerable victims — the state must act as guardian.
 - **Rule of Law**: Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.
   - Application to this case: Foundational principle engaged in every challenge to executive or legislative action.
 ### VII. PRIORITY ASSESSMENT &amp; JUSTIFICATION
-**Assigned Priority:** Medium
-**Category Rationale:** Company law matters involve corporate governance, shareholder rights, and commercial disputes. While they can have significant economic consequences affecting livelihoods (Article 21), they do not involve direct threats to life or physical safety. They warrant moderated priority unless fraud, criminal conduct, or imminent liquidation threatening employee welfare is established.
+**Assigned Priority:** High
+**Category Rationale:** Cases involving violent crime directly implicate the most fundamental right under the Constitution — the right to life. The state's failure to accord such cases the highest priority would constitute a violation of its affirmative obligation under Article 21 to protect life and ensure access to justice.
 ### VIII. FINAL OBSERVATION
-From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **Medium Priority**. 
-The case presents meaningful legal or constitutional issues that warrant attentive but not extraordinary expedition. The court should monitor the progress of this matter to ensure it does not languish, while recognising that cases involving imminent threats to life or liberty must take precedence.</t>
+From the perspective of an unbiased state adjudicating under the Constitution of India, this matter has been assigned **High Priority**. 
+This is constitutionally appropriate and reflects the gravity of the rights engaged. The court is directed to list this matter expeditiously, ensuring that no procedural delay undermines the constitutional rights at stake. The State must accord this case the attention and resources commensurate with its priority level.</t>
   </si>
   <si>
     <t>**RULE 1 — No Physical Injury → Standard Priority:** Article 21 (right to life) is not directly engaged through physical harm. Priority is determined by other factors.
@@ -1096,6 +1100,13 @@
 **FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **Medium**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
   </si>
   <si>
+    <t>**RULE 1 — Major Injury → High Priority (Article 21):** Bodily integrity and the right to health under Article 21 are seriously compromised. Strong urgency is constitutionally required.
+**RULE 2 — High Vulnerability → Elevated Priority (Doctrine of Parens Patriae):** The state has a special duty to protect vulnerable persons. Articles 15, 39, and 39A require the court to ensure that vulnerable litigants are not disadvantaged by delay.
+**RULE 3 — Power Imbalance → Ensure Level Playing Field (Article 14):** A significant power imbalance between parties triggers Article 14's equality guarantee. The court must take active measures to prevent the influential party from exploiting its position.
+**RULE 4 — Violent Crime → Article 21 Primacy:** Criminal matters involving violence directly implicate the right to life and personal liberty. The state's duty under Article 21 requires urgent judicial attention.
+**FINAL DETERMINATION:** Based on the above constitutional rules and the extracted case features, the priority assigned is **High**. This determination represents the impartial state's assessment of the urgency required to ensure that constitutional rights are protected and justice is delivered without undue delay.</t>
+  </si>
+  <si>
     <t>case_priority_system\decision_graphs\03_Exhibit_P2_Bank_Transfers_decision_report.md</t>
   </si>
   <si>
@@ -1147,6 +1158,9 @@
     <t>Medium</t>
   </si>
   <si>
+    <t>High</t>
+  </si>
+  <si>
     <t>Excise/Tax</t>
   </si>
   <si>
@@ -1156,16 +1170,19 @@
     <t>Constitutional/Writ</t>
   </si>
   <si>
-    <t>Company/Winding Up</t>
+    <t>Criminal/Violent</t>
   </si>
   <si>
     <t>Non-Violent</t>
   </si>
   <si>
+    <t>Violent</t>
+  </si>
+  <si>
     <t>No Injury</t>
   </si>
   <si>
-    <t>High</t>
+    <t>Major</t>
   </si>
   <si>
     <t>[{'article': 'Article 265', 'title': 'Tax Not to be Imposed Save by Authority of Law', 'primary': True, 'why_applies': 'This is a tax case. Article 265 says the government cannot collect any tax unless a law specifically allows it. If the tax was charged without proper legal backing, it must be given back.', 'precedents': []}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other.', 'precedents': []}, {'article': 'Article 19(1)(g)', 'title': 'Right to Practise Any Profession or Carry On Occupation, Trade or Business', 'primary': True, 'why_applies': "This case is about someone's right to run a business, practice a trade, or do a job. Article 19(1)(g) protects that right, but the government can put fair limits on it if the public interest requires it. The court must decide if those limits were reasonable.", 'precedents': []}, {'article': 'Article 300A', 'title': 'Right to Property', 'primary': False, 'why_applies': 'This case involves property or money. Article 300A protects people from losing their property without a lawful reason. The court must check that the proper legal process was followed.', 'precedents': []}, {'article': 'Article 301', 'title': 'Freedom of Trade, Commerce and Intercourse', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': False, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason.", 'precedents': []}]</t>
@@ -1189,7 +1206,7 @@
     <t>[{'article': 'Article 265', 'title': 'Tax Not to be Imposed Save by Authority of Law', 'primary': True, 'why_applies': 'This is a tax case. Article 265 says the government cannot collect any tax unless a law specifically allows it. If the tax was charged without proper legal backing, it must be given back.', 'precedents': []}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other. A vulnerable person is involved — like a child, an elderly person, or someone from a disadvantaged community. The government has a special duty to protect them. One side is much more powerful than the other — a government body, a large company, or someone with political influence. Article 14 requires the court to make sure the weaker party is not overpowered.', 'precedents': []}, {'article': 'Article 19(1)(g)', 'title': 'Right to Practise Any Profession or Carry On Occupation, Trade or Business', 'primary': True, 'why_applies': "This case is about someone's right to run a business, practice a trade, or do a job. Article 19(1)(g) protects that right, but the government can put fair limits on it if the public interest requires it. The court must decide if those limits were reasonable.", 'precedents': []}, {'article': 'Article 300A', 'title': 'Right to Property', 'primary': False, 'why_applies': 'This case involves property or money. Article 300A protects people from losing their property without a lawful reason. The court must check that the proper legal process was followed.', 'precedents': []}, {'article': 'Article 301', 'title': 'Freedom of Trade, Commerce and Intercourse', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': False, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason. A vulnerable person is involved — like a child, an elderly person, or someone from a disadvantaged community. The government has a special duty to protect them.", 'precedents': []}]</t>
   </si>
   <si>
-    <t>[{'article': 'Article 14', 'title': 'Equality Before Law', 'primary': True, 'why_applies': 'Article 14 means the law must treat everyone equally. This case involves a disagreement between two sides, and both sides deserve a fair chance to be heard. The judge must not favour one over the other. One side is much more powerful than the other — a government body, a large company, or someone with political influence. Article 14 requires the court to make sure the weaker party is not overpowered.', 'precedents': []}, {'article': 'Article 300A', 'title': 'Right to Property', 'primary': True, 'why_applies': 'This case involves property or money. Article 300A protects people from losing their property without a lawful reason. The court must check that the proper legal process was followed.', 'precedents': []}, {'article': 'Article 19(1)(g)', 'title': 'Right to Practise Any Profession or Carry On Occupation, Trade or Business', 'primary': True, 'why_applies': "This case is about someone's right to run a business, practice a trade, or do a job. Article 19(1)(g) protects that right, but the government can put fair limits on it if the public interest requires it. The court must decide if those limits were reasonable.", 'precedents': []}, {'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': False, 'why_applies': "Article 21 protects every person's right to life and freedom. It applies here because this case could affect someone's safety, freedom, or basic dignity. Even without physical harm, the court must make sure no one is deprived of their freedom without a valid reason.", 'precedents': []}, {'article': 'Article 39', 'title': 'Certain Principles of Policy to be Followed by the State', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 39A', 'title': 'Equal Justice and Free Legal Aid', 'primary': False, 'why_applies': '', 'precedents': []}]</t>
+    <t>[{'article': 'Article 21', 'title': 'Protection of Life and Personal Liberty', 'primary': True, 'why_applies': 'Someone has been badly hurt or their life is in danger. Article 21 says every person has the right to live with dignity. When someone is seriously injured, the government must act fast — make sure they get medical help and hold the person responsible for the harm. A vulnerable person is involved — like a child, an elderly person, or someone from a disadvantaged community. The government has a special duty to protect them.', 'precedents': []}, {'article': 'Article 22', 'title': 'Protection Against Arrest and Detention', 'primary': True, 'why_applies': 'Someone has been arrested. Article 22 says they must be told why, allowed to talk to a lawyer, and not kept in jail forever without a proper hearing. It protects people from being locked up without reason.', 'precedents': []}, {'article': 'Article 20', 'title': 'Protection in Respect of Conviction for Offences', 'primary': True, 'why_applies': 'This is a criminal case. Article 20 protects the accused person from being treated unfairly. It says: you cannot be punished for something that was not a crime when you did it, you cannot be tried twice for the same offence, and you cannot be forced to confess.', 'precedents': []}, {'article': 'Article 14', 'title': 'Equality Before Law', 'primary': False, 'why_applies': 'This is a criminal case. Article 14 says everyone must be treated the same way by the law — the person accused and the victim both deserve to be treated fairly. The court cannot take sides based on who someone is. A vulnerable person is involved — like a child, an elderly person, or someone from a disadvantaged community. The government has a special duty to protect them. One side is much more powerful than the other — a government body, a large company, or someone with political influence. Article 14 requires the court to make sure the weaker party is not overpowered.', 'precedents': []}, {'article': 'Article 17', 'title': 'Abolition of Untouchability', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 23', 'title': 'Prohibition of Traffic in Human Beings and Forced Labour', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 24', 'title': 'Prohibition of Employment of Children in Factories', 'primary': False, 'why_applies': '', 'precedents': []}, {'article': 'Article 39A', 'title': 'Equal Justice and Free Legal Aid', 'primary': False, 'why_applies': '', 'precedents': []}]</t>
   </si>
   <si>
     <t>Under Article 265, the State cannot levy or collect tax without the authority of law. The judiciary must ensure that tax proceedings are conducted lawfully, non-arbitrarily, and in accordance with principles of natural justice. The state's duty extends to ensuring that tax demands and assessments follow procedural fairness and that the citizen's right to carry on business (Article 19(1)(g)) is not unreasonably restricted.</t>
@@ -1201,7 +1218,7 @@
     <t>The State must ensure that all civil disputes are adjudicated fairly, transparently, and within a reasonable time. Under Article 14, the state guarantees equal access to justice — all litigants are entitled to a fair hearing. The principle of speedy trial (derived from Article 21) requires that even ordinary civil matters be resolved without inordinate delay, though they yield priority to cases involving life and liberty.</t>
   </si>
   <si>
-    <t>The State must ensure that company disputes and winding-up proceedings are adjudicated fairly, with due regard to the rights of shareholders, creditors, and employees. The judiciary must balance commercial efficiency with procedural fairness, ensuring that oppression and mismanagement claims are heard without undue delay but without displacing more urgent life-and-liberty matters.</t>
+    <t>The State has a non-derogable duty under Article 21 to protect the right to life and personal liberty of every person. In violent crimes, the judiciary must ensure: (a) immediate protection of the victim and witnesses, (b) preservation of evidence, (c) expeditious trial to prevent secondary victimisation, and (d) enforcement of the victim's right to a speedy trial as an integral part of Article 21.</t>
   </si>
   <si>
     <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}, {'name': 'Doctrine of Reasonable Classification', 'description': 'Article 14 permits classification of persons if it is based on intelligible differentia having a rational nexus with the object sought to be achieved.', 'application': 'Used to test whether differential treatment of litigants or groups is constitutional.'}]</t>
@@ -1211,6 +1228,9 @@
   </si>
   <si>
     <t>[{'name': 'Doctrine of Basic Structure', 'description': 'The Parliament cannot amend the Constitution to destroy its basic features such as supremacy of the Constitution, rule of law, and judicial review.', 'application': 'Applicable to cases involving constitutional amendments or executive actions affecting foundational principles.'}, {'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Principle of Natural Justice — Audi Alteram Partem', 'description': 'No person shall be condemned without being heard. The right to be heard is a fundamental principle of justice.', 'application': 'Ensures procedural fairness in administrative and quasi-judicial proceedings.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}, {'name': 'Doctrine of Colourable Legislation', 'description': 'If the legislature lacks the competence to enact a law directly, it cannot do indirectly what it cannot do directly — such camouflage is struck down.', 'application': 'Applicable where a statute purports to do one thing but in substance does another outside legislative competence.'}, {'name': 'Doctrine of Harmonious Construction', 'description': 'Where two constitutional provisions conflict, they should be interpreted so that both are given effect rather than one nullifying the other.', 'application': 'Used when Articles or statutory provisions appear to overlap or clash.'}]</t>
+  </si>
+  <si>
+    <t>[{'name': 'Doctrine of Proportionality', 'description': 'Any state action restricting rights must be proportionate to the aim sought — it must be necessary, suitable, and not excessive.', 'application': 'Used to assess whether the priority assigned is proportionate to the gravity of the rights violation.'}, {'name': 'Doctrine of Parens Patriae', 'description': 'The state has a duty to protect those who cannot protect themselves, such as minors, disabled persons, and the mentally ill.', 'application': 'Critical for cases involving vulnerable victims — the state must act as guardian.'}, {'name': 'Rule of Law', 'description': 'Every person, including the State, is subject to the law; no one is above it. Government action must have legal authority.', 'application': 'Foundational principle engaged in every challenge to executive or legislative action.'}]</t>
   </si>
   <si>
     <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
@@ -1246,9 +1266,11 @@
 **Category-Specific Analysis — Excise/Tax:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
   </si>
   <si>
-    <t>**Primary Interest — Other Constitutional Rights:** With severity 'No Injury', the primary constitutional concern shifts from the right to life (Article 21) to other guarantees such as equality (Article 14), freedom of trade (Article 19(1)(g)), or property rights (Article 300A) as applicable. While these rights are fundamental, they permit greater flexibility in prioritisation.
+    <t>**Primary Interest — Right to Life &amp; Bodily Integrity (Article 21):** The severity level 'Major' indicates that the right to life or physical integrity has been seriously compromised. Under Article 21, this is the weightiest constitutional interest and must take precedence over all other considerations. The state's duty to protect life is non-derogable and non-delegable.
+**Assessment:** The High priority correctly reflects the primacy of Article 21 rights. This is constitutionally appropriate and proportionate to the gravity of the harm.
+**Vulnerability Analysis — Special State Obligation:** A vulnerable party is involved. The Doctrine of Parens Patriae and Articles 15(3), 15(4), 39, and 39A impose a heightened duty on the state to protect the vulnerable. This factor strongly supports High priority to prevent further harm or injustice.
 **Power Imbalance — Article 14 Equality Concern:** There is a significant power imbalance between the parties. Article 14 requires the state to ensure equality before the law. Where one party is a government body, large corporation, or influential entity, the court must guard against the risk that institutional power could subvert the fairness of proceedings. The assigned priority adequately accounts for this concern.
-**Category-Specific Analysis — Company/Winding Up:** This is primarily a regulatory/commercial matter. While Article 14 equality and Article 300A property rights are engaged, the case does not involve the same constitutional urgency as life-and-liberty cases. The assigned priority appropriately reflects this proportionally.</t>
+**Category-Specific Analysis — Criminal/Violent:** This category involves the most serious engagement of constitutional rights — the right to life, liberty, and safety of persons. The High priority assigned is constitutionally mandated.</t>
   </si>
   <si>
     <t>case_priority_system\reports\03_Exhibit_P2_Bank_Transfers_report.pdf</t>
@@ -1722,46 +1744,46 @@
         <v>79</v>
       </c>
       <c r="F2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="L2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="N2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="P2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="Q2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="R2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="S2" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="T2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1781,46 +1803,46 @@
         <v>79</v>
       </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="L3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="N3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="P3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="Q3" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="R3" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="S3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="T3" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1840,46 +1862,46 @@
         <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="L4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="N4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="P4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="Q4" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="R4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="S4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="T4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1899,46 +1921,46 @@
         <v>81</v>
       </c>
       <c r="F5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H5" t="s">
+        <v>103</v>
+      </c>
+      <c r="I5" t="s">
+        <v>105</v>
+      </c>
+      <c r="J5" t="s">
+        <v>109</v>
+      </c>
+      <c r="K5" t="s">
+        <v>111</v>
+      </c>
+      <c r="L5" t="s">
         <v>102</v>
       </c>
-      <c r="I5" t="s">
-        <v>103</v>
-      </c>
-      <c r="J5" t="s">
-        <v>107</v>
-      </c>
-      <c r="K5" t="s">
-        <v>108</v>
-      </c>
-      <c r="L5" t="s">
-        <v>101</v>
-      </c>
       <c r="M5" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="N5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="P5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="Q5" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="R5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="S5" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="T5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -1958,46 +1980,46 @@
         <v>79</v>
       </c>
       <c r="F6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K6" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="L6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="N6" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="P6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="Q6" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="R6" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="S6" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="T6" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -2017,46 +2039,46 @@
         <v>82</v>
       </c>
       <c r="F7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H7" t="s">
+        <v>103</v>
+      </c>
+      <c r="I7" t="s">
+        <v>107</v>
+      </c>
+      <c r="J7" t="s">
+        <v>109</v>
+      </c>
+      <c r="K7" t="s">
+        <v>111</v>
+      </c>
+      <c r="L7" t="s">
         <v>102</v>
       </c>
-      <c r="I7" t="s">
-        <v>105</v>
-      </c>
-      <c r="J7" t="s">
-        <v>107</v>
-      </c>
-      <c r="K7" t="s">
-        <v>108</v>
-      </c>
-      <c r="L7" t="s">
-        <v>101</v>
-      </c>
       <c r="M7" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="N7" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="P7" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="Q7" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="R7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="S7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="T7" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -2076,49 +2098,49 @@
         <v>81</v>
       </c>
       <c r="F8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H8" t="s">
+        <v>103</v>
+      </c>
+      <c r="I8" t="s">
+        <v>105</v>
+      </c>
+      <c r="J8" t="s">
+        <v>109</v>
+      </c>
+      <c r="K8" t="s">
+        <v>111</v>
+      </c>
+      <c r="L8" t="s">
         <v>102</v>
       </c>
-      <c r="I8" t="s">
-        <v>103</v>
-      </c>
-      <c r="J8" t="s">
-        <v>107</v>
-      </c>
-      <c r="K8" t="s">
-        <v>108</v>
-      </c>
-      <c r="L8" t="s">
-        <v>101</v>
-      </c>
       <c r="M8" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="N8" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="O8" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="P8" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="Q8" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="R8" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="S8" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="T8" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -2138,49 +2160,49 @@
         <v>83</v>
       </c>
       <c r="F9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="J9" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K9" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="L9" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="M9" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="N9" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="O9" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="P9" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="Q9" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="R9" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="S9" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="T9" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -2200,49 +2222,49 @@
         <v>82</v>
       </c>
       <c r="F10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H10" t="s">
+        <v>103</v>
+      </c>
+      <c r="I10" t="s">
+        <v>107</v>
+      </c>
+      <c r="J10" t="s">
+        <v>109</v>
+      </c>
+      <c r="K10" t="s">
+        <v>111</v>
+      </c>
+      <c r="L10" t="s">
         <v>102</v>
       </c>
-      <c r="I10" t="s">
-        <v>105</v>
-      </c>
-      <c r="J10" t="s">
-        <v>107</v>
-      </c>
-      <c r="K10" t="s">
-        <v>108</v>
-      </c>
-      <c r="L10" t="s">
-        <v>101</v>
-      </c>
       <c r="M10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="N10" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="O10" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="P10" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="Q10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="R10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="S10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="T10" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -2262,49 +2284,49 @@
         <v>84</v>
       </c>
       <c r="F11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I11" t="s">
+        <v>106</v>
+      </c>
+      <c r="J11" t="s">
+        <v>109</v>
+      </c>
+      <c r="K11" t="s">
+        <v>111</v>
+      </c>
+      <c r="L11" t="s">
         <v>102</v>
       </c>
-      <c r="I11" t="s">
+      <c r="M11" t="s">
         <v>104</v>
       </c>
-      <c r="J11" t="s">
-        <v>107</v>
-      </c>
-      <c r="K11" t="s">
-        <v>108</v>
-      </c>
-      <c r="L11" t="s">
-        <v>101</v>
-      </c>
-      <c r="M11" t="s">
-        <v>109</v>
-      </c>
       <c r="N11" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O11" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="P11" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="Q11" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="R11" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="S11" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="T11" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -2324,49 +2346,49 @@
         <v>83</v>
       </c>
       <c r="F12" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G12" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I12" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="J12" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K12" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="L12" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="M12" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="N12" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="O12" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="P12" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="Q12" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="R12" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="S12" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="T12" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -2386,49 +2408,49 @@
         <v>82</v>
       </c>
       <c r="F13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H13" t="s">
+        <v>103</v>
+      </c>
+      <c r="I13" t="s">
+        <v>107</v>
+      </c>
+      <c r="J13" t="s">
+        <v>109</v>
+      </c>
+      <c r="K13" t="s">
+        <v>111</v>
+      </c>
+      <c r="L13" t="s">
         <v>102</v>
       </c>
-      <c r="I13" t="s">
-        <v>105</v>
-      </c>
-      <c r="J13" t="s">
-        <v>107</v>
-      </c>
-      <c r="K13" t="s">
-        <v>108</v>
-      </c>
-      <c r="L13" t="s">
-        <v>101</v>
-      </c>
       <c r="M13" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="N13" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="O13" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="P13" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="Q13" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="R13" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="S13" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="T13" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -2448,49 +2470,49 @@
         <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I14" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J14" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K14" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="L14" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="M14" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="N14" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="O14" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="P14" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="Q14" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="R14" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="S14" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="T14" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -2510,49 +2532,49 @@
         <v>82</v>
       </c>
       <c r="F15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H15" t="s">
+        <v>103</v>
+      </c>
+      <c r="I15" t="s">
+        <v>107</v>
+      </c>
+      <c r="J15" t="s">
+        <v>109</v>
+      </c>
+      <c r="K15" t="s">
+        <v>111</v>
+      </c>
+      <c r="L15" t="s">
         <v>102</v>
       </c>
-      <c r="I15" t="s">
-        <v>105</v>
-      </c>
-      <c r="J15" t="s">
-        <v>107</v>
-      </c>
-      <c r="K15" t="s">
-        <v>108</v>
-      </c>
-      <c r="L15" t="s">
-        <v>101</v>
-      </c>
       <c r="M15" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="N15" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="O15" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="P15" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="Q15" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="R15" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="S15" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="T15" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -2569,52 +2591,52 @@
         <v>78</v>
       </c>
       <c r="E16" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H16" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I16" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="J16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="K16" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="L16" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="M16" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="N16" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="O16" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="P16" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="Q16" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="R16" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="S16" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="T16" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>